<commit_message>
Apply strict no-government-ownership rule and split files by category
Drop Enova, G4S UAE, ServeU and Dulsco (government or state
shareholders, incl. partial/indirect). Add Al-Futtaim Engineering FM,
Al Naboodah FM, AJAD FM and Al Manal Security. Add a government
ownership check column and separate FM, Security and Cleaning files.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01QTLqykBaXLnYN7UB8pKnAZ
</commit_message>
<xml_diff>
--- a/research/mebs-competitors/MEBS_Competitors_UAE.xlsx
+++ b/research/mebs-competitors/MEBS_Competitors_UAE.xlsx
@@ -15,9 +15,9 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Excluded (gov-linked)" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'FM Companies'!$A$1:$R$9</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Security Only'!$A$1:$R$7</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Cleaning Only'!$A$1:$R$7</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'FM Companies'!$A$1:$S$9</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Security Only'!$A$1:$S$7</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Cleaning Only'!$A$1:$S$7</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -511,7 +511,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Prepared 30 Oct 2026 from public web sources. Government-owned or government-linked companies are excluded (see 'Excluded' sheet).</t>
+          <t>Prepared 30 Oct 2026 from public web sources. Rule: no company with a government or state owner, including partial or indirect stakes (see 'Excluded' sheet).</t>
         </is>
       </c>
     </row>
@@ -528,7 +528,8 @@
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>1. FM Companies (8)  2. Security Only (6)  3. Cleaning Only (6)  4. MEBS benchmark  5. Excluded (gov-linked)</t>
+          <t>1. FM Companies (8)  2. Security Only (6)  3. Cleaning Only (6)  4. MEBS benchmark  5. Excluded (gov-linked)
+Separate files are also provided per category.</t>
         </is>
       </c>
     </row>
@@ -595,7 +596,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R9"/>
+  <dimension ref="A1:S9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="4" customWidth="1" min="1" max="1"/>
@@ -614,8 +615,9 @@
     <col width="22" customWidth="1" min="14" max="14"/>
     <col width="30" customWidth="1" min="15" max="15"/>
     <col width="34" customWidth="1" min="16" max="16"/>
-    <col width="12" customWidth="1" min="17" max="17"/>
-    <col width="46" customWidth="1" min="18" max="18"/>
+    <col width="28" customWidth="1" min="17" max="17"/>
+    <col width="12" customWidth="1" min="18" max="18"/>
+    <col width="46" customWidth="1" min="19" max="19"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -701,10 +703,15 @@
       </c>
       <c r="Q1" s="4" t="inlineStr">
         <is>
+          <t>Government ownership check</t>
+        </is>
+      </c>
+      <c r="R1" s="4" t="inlineStr">
+        <is>
           <t>Data confidence</t>
         </is>
       </c>
-      <c r="R1" s="4" t="inlineStr">
+      <c r="S1" s="4" t="inlineStr">
         <is>
           <t>Main sources</t>
         </is>
@@ -791,10 +798,15 @@
       </c>
       <c r="Q2" s="5" t="inlineStr">
         <is>
+          <t>No government or state shareholder found in public sources</t>
+        </is>
+      </c>
+      <c r="R2" s="5" t="inlineStr">
+        <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="R2" s="5" t="inlineStr">
+      <c r="S2" s="5" t="inlineStr">
         <is>
           <t>farnek.com/about-us; thenationalnews.com (Oberlin profile); farnek.com (AED 607M 2023 release); i-fm.net (Dubai Airports)</t>
         </is>
@@ -881,10 +893,15 @@
       </c>
       <c r="Q3" s="5" t="inlineStr">
         <is>
+          <t>Private shareholders (names not published); bought out EMCOR in 2009. No government stake found</t>
+        </is>
+      </c>
+      <c r="R3" s="5" t="inlineStr">
+        <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="R3" s="5" t="inlineStr">
+      <c r="S3" s="5" t="inlineStr">
         <is>
           <t>forbesmiddleeast.com (Tariq Chauhan); gulfbusiness.com (EMCOR buyout); zawya.com (SecurePlus, Guardian acquisitions); newsroom.efsme.com</t>
         </is>
@@ -896,87 +913,92 @@
       </c>
       <c r="B4" s="6" t="inlineStr">
         <is>
-          <t>Enova by Veolia</t>
+          <t>Al Shirawi Facilities Management LLC</t>
         </is>
       </c>
       <c r="C4" s="5" t="inlineStr">
         <is>
-          <t>Facility &amp; energy management: MEP, soft services, energy performance contracts (Hubgrade monitoring centre)</t>
+          <t>Integrated FM: MEP, civil, cleaning, landscaping, pest control</t>
         </is>
       </c>
       <c r="D4" s="5" t="inlineStr">
         <is>
-          <t>JV: Majid Al Futtaim (private Emirati family conglomerate) + Veolia (French, listed)</t>
+          <t>Al Shirawi Group. Chairman Mohamed Al Shirawi; co-founders Abdulla Al Shirawi and Mohan Valrani</t>
         </is>
       </c>
       <c r="E4" s="5" t="inlineStr">
         <is>
-          <t>Emirati / French</t>
+          <t>Emirati / Indian</t>
         </is>
       </c>
       <c r="F4" s="5" t="inlineStr">
         <is>
-          <t>Private JV</t>
+          <t>Private family group</t>
         </is>
       </c>
       <c r="G4" s="5" t="inlineStr">
         <is>
-          <t>2002</t>
+          <t>Group 1971 (FM operations from 1974 per MEFMA listing)</t>
         </is>
       </c>
       <c r="H4" s="5" t="inlineStr">
         <is>
-          <t>Deira City Centre complex, Dubai</t>
+          <t>Dubai</t>
         </is>
       </c>
       <c r="I4" s="5" t="inlineStr">
         <is>
-          <t>UAE, KSA, Egypt, Oman, Qatar, Türkiye</t>
+          <t>UAE</t>
         </is>
       </c>
       <c r="J4" s="5" t="inlineStr">
         <is>
-          <t>3,000+ (company)</t>
+          <t>1,500+ (FM company, 2016); Group 10,500 to 11,000</t>
         </is>
       </c>
       <c r="K4" s="5" t="inlineStr">
         <is>
-          <t>Malls and retail portfolios; Hubgrade remote energy monitoring centre</t>
+          <t>Part of 30+ company group; awards from RTA; ISO 41001 (BSI); BICSc certified</t>
         </is>
       </c>
       <c r="L4" s="5" t="inlineStr">
         <is>
-          <t>Not published (third-party estimates unreliable)</t>
+          <t>Not published</t>
         </is>
       </c>
       <c r="M4" s="5" t="inlineStr">
         <is>
-          <t>approx. AED 225M to 330M</t>
+          <t>approx. AED 112M to 220M</t>
         </is>
       </c>
       <c r="N4" s="5" t="inlineStr">
         <is>
-          <t>ISO-certified (per company)</t>
+          <t>ISO 41001, BICSc</t>
         </is>
       </c>
       <c r="O4" s="5" t="inlineStr">
         <is>
-          <t>MAF malls (City Centre, Mall of the Emirates), Dubai Airports Emiratisation partnership, Saudi malls</t>
+          <t>Dubai Design District, Dubai International Humanitarian City, RTA, IT Plaza (HOAM)</t>
         </is>
       </c>
       <c r="P4" s="5" t="inlineStr">
         <is>
-          <t>Strong in retail, mall and commercial FM where MEBS sells security and cleaning</t>
+          <t>Private Emirati-backed Dubai IFM, similar commercial/community client base</t>
         </is>
       </c>
       <c r="Q4" s="5" t="inlineStr">
         <is>
+          <t>No government or state shareholder found in public sources</t>
+        </is>
+      </c>
+      <c r="R4" s="5" t="inlineStr">
+        <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="R4" s="5" t="inlineStr">
-        <is>
-          <t>enova-me.com; Enova corporate brochure (emiratesgbc.org); zawya.com (Saudi malls contract)</t>
+      <c r="S4" s="5" t="inlineStr">
+        <is>
+          <t>mefma.org (Al Shirawi FM); zawya.com (d3, ISO 41001 releases); wikipedia (Mohan Valrani); entrepreneur.com</t>
         </is>
       </c>
     </row>
@@ -986,22 +1008,22 @@
       </c>
       <c r="B5" s="6" t="inlineStr">
         <is>
-          <t>Al Shirawi Facilities Management LLC</t>
+          <t>INAYA Facilities Management Services</t>
         </is>
       </c>
       <c r="C5" s="5" t="inlineStr">
         <is>
-          <t>Integrated FM: MEP, civil, cleaning, landscaping, pest control</t>
+          <t>Integrated FM: MEP, cleaning, soft services, helpdesk</t>
         </is>
       </c>
       <c r="D5" s="5" t="inlineStr">
         <is>
-          <t>Al Shirawi Group. Chairman Mohamed Al Shirawi; co-founders Abdulla Al Shirawi and Mohan Valrani</t>
+          <t>Belhasa Group. Chairman Ahmed Saif Belhasa</t>
         </is>
       </c>
       <c r="E5" s="5" t="inlineStr">
         <is>
-          <t>Emirati / Indian</t>
+          <t>Emirati</t>
         </is>
       </c>
       <c r="F5" s="5" t="inlineStr">
@@ -1011,7 +1033,7 @@
       </c>
       <c r="G5" s="5" t="inlineStr">
         <is>
-          <t>Group 1971 (FM operations from 1974 per MEFMA listing)</t>
+          <t>December 2010</t>
         </is>
       </c>
       <c r="H5" s="5" t="inlineStr">
@@ -1021,17 +1043,17 @@
       </c>
       <c r="I5" s="5" t="inlineStr">
         <is>
-          <t>UAE</t>
+          <t>UAE, wider GCC</t>
         </is>
       </c>
       <c r="J5" s="5" t="inlineStr">
         <is>
-          <t>1,500+ (FM company, 2016); Group 10,500 to 11,000</t>
+          <t>501 to 1,000 (aggregator, unverified)</t>
         </is>
       </c>
       <c r="K5" s="5" t="inlineStr">
         <is>
-          <t>Part of 30+ company group; awards from RTA; ISO 41001 (BSI); BICSc certified</t>
+          <t>Mall and commercial portfolios</t>
         </is>
       </c>
       <c r="L5" s="5" t="inlineStr">
@@ -1041,32 +1063,37 @@
       </c>
       <c r="M5" s="5" t="inlineStr">
         <is>
-          <t>approx. AED 112M to 220M</t>
+          <t>approx. AED 38M to 110M</t>
         </is>
       </c>
       <c r="N5" s="5" t="inlineStr">
         <is>
-          <t>ISO 41001, BICSc</t>
+          <t>ISO 14001, OHSAS 18001 (2014)</t>
         </is>
       </c>
       <c r="O5" s="5" t="inlineStr">
         <is>
-          <t>Dubai Design District, Dubai International Humanitarian City, RTA, IT Plaza (HOAM)</t>
+          <t>Ibn Battuta Mall</t>
         </is>
       </c>
       <c r="P5" s="5" t="inlineStr">
         <is>
-          <t>Private Emirati-backed Dubai IFM, similar commercial/community client base</t>
+          <t>Closest size peer to MEBS; Emirati family-owned Dubai IFM</t>
         </is>
       </c>
       <c r="Q5" s="5" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>No government or state shareholder found in public sources</t>
         </is>
       </c>
       <c r="R5" s="5" t="inlineStr">
         <is>
-          <t>mefma.org (Al Shirawi FM); zawya.com (d3, ISO 41001 releases); wikipedia (Mohan Valrani); entrepreneur.com</t>
+          <t>Low to medium</t>
+        </is>
+      </c>
+      <c r="S5" s="5" t="inlineStr">
+        <is>
+          <t>gulfnews.com (INAYA launch); zawya.com (ISO award, Ibn Battuta); prospeo.io</t>
         </is>
       </c>
     </row>
@@ -1076,32 +1103,32 @@
       </c>
       <c r="B6" s="6" t="inlineStr">
         <is>
-          <t>INAYA Facilities Management Services</t>
+          <t>Delight International Facilities Management LLC</t>
         </is>
       </c>
       <c r="C6" s="5" t="inlineStr">
         <is>
-          <t>Integrated FM: MEP, cleaning, soft services, helpdesk</t>
+          <t>Integrated FM: cleaning (origin), MEP maintenance, soft services</t>
         </is>
       </c>
       <c r="D6" s="5" t="inlineStr">
         <is>
-          <t>Belhasa Group. Chairman Ahmed Saif Belhasa</t>
+          <t>Private (Delight group of companies). Owner name not published</t>
         </is>
       </c>
       <c r="E6" s="5" t="inlineStr">
         <is>
-          <t>Emirati</t>
+          <t>Not published</t>
         </is>
       </c>
       <c r="F6" s="5" t="inlineStr">
         <is>
-          <t>Private family group</t>
+          <t>Private</t>
         </is>
       </c>
       <c r="G6" s="5" t="inlineStr">
         <is>
-          <t>December 2010</t>
+          <t>1991</t>
         </is>
       </c>
       <c r="H6" s="5" t="inlineStr">
@@ -1111,17 +1138,17 @@
       </c>
       <c r="I6" s="5" t="inlineStr">
         <is>
-          <t>UAE, wider GCC</t>
+          <t>Dubai, Abu Dhabi</t>
         </is>
       </c>
       <c r="J6" s="5" t="inlineStr">
         <is>
-          <t>501 to 1,000 (aggregator, unverified)</t>
+          <t>500+ (company)</t>
         </is>
       </c>
       <c r="K6" s="5" t="inlineStr">
         <is>
-          <t>Mall and commercial portfolios</t>
+          <t>Started as a cleaning company and grew into IFM</t>
         </is>
       </c>
       <c r="L6" s="5" t="inlineStr">
@@ -1131,32 +1158,37 @@
       </c>
       <c r="M6" s="5" t="inlineStr">
         <is>
-          <t>approx. AED 38M to 110M</t>
+          <t>approx. AED 38M to 77M</t>
         </is>
       </c>
       <c r="N6" s="5" t="inlineStr">
         <is>
-          <t>ISO 14001, OHSAS 18001 (2014)</t>
+          <t>ISO certified (per company)</t>
         </is>
       </c>
       <c r="O6" s="5" t="inlineStr">
         <is>
-          <t>Ibn Battuta Mall</t>
+          <t>Not published</t>
         </is>
       </c>
       <c r="P6" s="5" t="inlineStr">
         <is>
-          <t>Closest size peer to MEBS; Emirati family-owned Dubai IFM</t>
+          <t>Size peer that also grew from one service line into IFM, as MEBS did</t>
         </is>
       </c>
       <c r="Q6" s="5" t="inlineStr">
         <is>
-          <t>Low to medium</t>
+          <t>No government or state shareholder found in public sources</t>
         </is>
       </c>
       <c r="R6" s="5" t="inlineStr">
         <is>
-          <t>gulfnews.com (INAYA launch); zawya.com (ISO award, Ibn Battuta); prospeo.io</t>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="S6" s="5" t="inlineStr">
+        <is>
+          <t>delightifm.com/about; devex.com; enggpro.com</t>
         </is>
       </c>
     </row>
@@ -1166,87 +1198,92 @@
       </c>
       <c r="B7" s="6" t="inlineStr">
         <is>
-          <t>Delight International Facilities Management LLC</t>
+          <t>Al-Futtaim Engineering &amp; Technologies (Facilities Management division)</t>
         </is>
       </c>
       <c r="C7" s="5" t="inlineStr">
         <is>
-          <t>Integrated FM: cleaning (origin), MEP maintenance, soft services</t>
+          <t>Facilities maintenance (MEP, civil), property strategy, infrastructure and golf course maintenance, outsourced technical manpower</t>
         </is>
       </c>
       <c r="D7" s="5" t="inlineStr">
         <is>
-          <t>Private (Delight group of companies). Owner name not published</t>
+          <t>Al-Futtaim Group (Al-Futtaim family). Chairman Omar Al-Futtaim</t>
         </is>
       </c>
       <c r="E7" s="5" t="inlineStr">
         <is>
+          <t>Emirati</t>
+        </is>
+      </c>
+      <c r="F7" s="5" t="inlineStr">
+        <is>
+          <t>Private family group</t>
+        </is>
+      </c>
+      <c r="G7" s="5" t="inlineStr">
+        <is>
+          <t>Group 1930s; FM division part of Al-Futtaim Engineering</t>
+        </is>
+      </c>
+      <c r="H7" s="5" t="inlineStr">
+        <is>
+          <t>Dubai</t>
+        </is>
+      </c>
+      <c r="I7" s="5" t="inlineStr">
+        <is>
+          <t>UAE, Qatar</t>
+        </is>
+      </c>
+      <c r="J7" s="5" t="inlineStr">
+        <is>
+          <t>Not published for FM division (Al-Futtaim Group approx. 42,000)</t>
+        </is>
+      </c>
+      <c r="K7" s="5" t="inlineStr">
+        <is>
+          <t>Part of a 200+ company private group</t>
+        </is>
+      </c>
+      <c r="L7" s="5" t="inlineStr">
+        <is>
           <t>Not published</t>
         </is>
       </c>
-      <c r="F7" s="5" t="inlineStr">
-        <is>
-          <t>Private</t>
-        </is>
-      </c>
-      <c r="G7" s="5" t="inlineStr">
-        <is>
-          <t>1991</t>
-        </is>
-      </c>
-      <c r="H7" s="5" t="inlineStr">
-        <is>
-          <t>Dubai</t>
-        </is>
-      </c>
-      <c r="I7" s="5" t="inlineStr">
-        <is>
-          <t>Dubai, Abu Dhabi</t>
-        </is>
-      </c>
-      <c r="J7" s="5" t="inlineStr">
-        <is>
-          <t>500+ (company)</t>
-        </is>
-      </c>
-      <c r="K7" s="5" t="inlineStr">
-        <is>
-          <t>Started as a cleaning company and grew into IFM</t>
-        </is>
-      </c>
-      <c r="L7" s="5" t="inlineStr">
+      <c r="M7" s="5" t="inlineStr">
+        <is>
+          <t>Cannot estimate (headcount unknown)</t>
+        </is>
+      </c>
+      <c r="N7" s="5" t="inlineStr">
         <is>
           <t>Not published</t>
         </is>
       </c>
-      <c r="M7" s="5" t="inlineStr">
-        <is>
-          <t>approx. AED 38M to 77M</t>
-        </is>
-      </c>
-      <c r="N7" s="5" t="inlineStr">
-        <is>
-          <t>ISO certified (per company)</t>
-        </is>
-      </c>
       <c r="O7" s="5" t="inlineStr">
         <is>
-          <t>Not published</t>
+          <t>Ministry of Education, Government of Sharjah, Dubai Municipality, dnata</t>
         </is>
       </c>
       <c r="P7" s="5" t="inlineStr">
         <is>
-          <t>Size peer that also grew from one service line into IFM, as MEBS did</t>
+          <t>Private Emirati engineering-led FM competitor for MEP and maintenance contracts</t>
         </is>
       </c>
       <c r="Q7" s="5" t="inlineStr">
         <is>
-          <t>Low</t>
+          <t>No government or state shareholder found in public sources</t>
         </is>
       </c>
       <c r="R7" s="5" t="inlineStr">
         <is>
-          <t>delightifm.com/about; devex.com; enggpro.com</t>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="S7" s="5" t="inlineStr">
+        <is>
+          <t>meconstructionnews.com (AFET MEFMA partner); zawya.com (AFET maintenance contracts); khaleejtimes.com</t>
         </is>
       </c>
     </row>
@@ -1256,17 +1293,17 @@
       </c>
       <c r="B8" s="6" t="inlineStr">
         <is>
-          <t>Dulsco Group</t>
+          <t>Al Naboodah Facilities Management</t>
         </is>
       </c>
       <c r="C8" s="5" t="inlineStr">
         <is>
-          <t>Manpower outsourcing (People Solutions), waste management (Environmental Solutions), FM services, recruitment</t>
+          <t>Integrated hard and soft FM: security, concierge, energy and waste management, pest control, water tank cleaning, landscaping, fire systems</t>
         </is>
       </c>
       <c r="D8" s="5" t="inlineStr">
         <is>
-          <t>Private shareholders incl. Sheikh Mana bin Khalifa Al Maktoum (founder WAFI Group, private capacity) and Abdul Rahman Sharif Al Baidhaei (ARMS Group). Group CEO David Stockton</t>
+          <t>Al Naboodah Group Enterprises (Al Naboodah family). Sits under Al Naboodah Construction Group (CEO Senan Al Naboodah)</t>
         </is>
       </c>
       <c r="E8" s="5" t="inlineStr">
@@ -1276,12 +1313,12 @@
       </c>
       <c r="F8" s="5" t="inlineStr">
         <is>
-          <t>Private (note: one shareholder is a royal family member in a private capacity, not a government entity)</t>
+          <t>Private family group</t>
         </is>
       </c>
       <c r="G8" s="5" t="inlineStr">
         <is>
-          <t>1935</t>
+          <t>Group 1958; FM unit launched as diversification (date not confirmed)</t>
         </is>
       </c>
       <c r="H8" s="5" t="inlineStr">
@@ -1291,27 +1328,27 @@
       </c>
       <c r="I8" s="5" t="inlineStr">
         <is>
-          <t>UAE, GCC, UK (acquired Advance Global Recruitment)</t>
+          <t>UAE</t>
         </is>
       </c>
       <c r="J8" s="5" t="inlineStr">
         <is>
-          <t>14,000+ (company)</t>
+          <t>Not published for FM unit (group approx. 32,000)</t>
         </is>
       </c>
       <c r="K8" s="5" t="inlineStr">
         <is>
-          <t>Workers deployed across 75 job categories; 90-year history</t>
+          <t>Fire and statutory services self-delivered within group</t>
         </is>
       </c>
       <c r="L8" s="5" t="inlineStr">
         <is>
-          <t>Not published (aggregator estimates range from US$400M to US$6.7B, unreliable)</t>
+          <t>Not published</t>
         </is>
       </c>
       <c r="M8" s="5" t="inlineStr">
         <is>
-          <t>approx. AED 1,050M to 1,540M</t>
+          <t>Cannot estimate (headcount unknown)</t>
         </is>
       </c>
       <c r="N8" s="5" t="inlineStr">
@@ -1321,22 +1358,27 @@
       </c>
       <c r="O8" s="5" t="inlineStr">
         <is>
-          <t>Large corporate and real estate clients</t>
+          <t>Group and third-party property portfolios</t>
         </is>
       </c>
       <c r="P8" s="5" t="inlineStr">
         <is>
-          <t>Supplies cleaning and FM manpower in the same Dubai market</t>
+          <t>Offers security + cleaning-type soft services alongside MEP, same model as MEBS</t>
         </is>
       </c>
       <c r="Q8" s="5" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>No government or state shareholder found in public sources</t>
         </is>
       </c>
       <c r="R8" s="5" t="inlineStr">
         <is>
-          <t>zawya.com (90 years release); khaleejtimes.com (AGR acquisition); gulftalent.com</t>
+          <t>Low to medium</t>
+        </is>
+      </c>
+      <c r="S8" s="5" t="inlineStr">
+        <is>
+          <t>gulfnews.com (Al Naboodah launches FM unit); technicalreviewmiddleeast.com; gulftalent.com</t>
         </is>
       </c>
     </row>
@@ -1346,62 +1388,62 @@
       </c>
       <c r="B9" s="6" t="inlineStr">
         <is>
-          <t>ServeU LLC</t>
+          <t>AJAD Facilities Management</t>
         </is>
       </c>
       <c r="C9" s="5" t="inlineStr">
         <is>
-          <t>Integrated FM: MEP, cleaning, housekeeping, disinfection, logistics; domestic workers unit</t>
+          <t>Total FM: MEP maintenance, cleaning, soft services</t>
         </is>
       </c>
       <c r="D9" s="5" t="inlineStr">
         <is>
-          <t>Union Properties PJSC (Dubai Financial Market listed; approx. 90% held by the general public)</t>
+          <t>100% Emirati-owned private company. Owner name not published</t>
         </is>
       </c>
       <c r="E9" s="5" t="inlineStr">
         <is>
-          <t>Emirati (listed parent)</t>
+          <t>Emirati</t>
         </is>
       </c>
       <c r="F9" s="5" t="inlineStr">
         <is>
-          <t>Subsidiary of a listed private-sector company</t>
+          <t>Private</t>
         </is>
       </c>
       <c r="G9" s="5" t="inlineStr">
         <is>
-          <t>1985</t>
+          <t>2002</t>
         </is>
       </c>
       <c r="H9" s="5" t="inlineStr">
         <is>
-          <t>Dubai</t>
+          <t>Abu Dhabi</t>
         </is>
       </c>
       <c r="I9" s="5" t="inlineStr">
         <is>
-          <t>UAE + 4 other countries</t>
+          <t>UAE</t>
         </is>
       </c>
       <c r="J9" s="5" t="inlineStr">
         <is>
-          <t>8,900+ (Gulf News)</t>
+          <t>Not reliably published (directory shows 30+)</t>
         </is>
       </c>
       <c r="K9" s="5" t="inlineStr">
         <is>
-          <t>Expo 2020 pavilions FM contracts (AED 18M); acquired House Keeping LLC for AED 100M</t>
+          <t>Residential, hospitality, healthcare, education and industrial clients</t>
         </is>
       </c>
       <c r="L9" s="5" t="inlineStr">
         <is>
-          <t>Not published separately (Union Properties H1 2025 revenue AED 316M, group level)</t>
+          <t>Not published</t>
         </is>
       </c>
       <c r="M9" s="5" t="inlineStr">
         <is>
-          <t>approx. AED 668M to 979M</t>
+          <t>Cannot estimate (headcount unknown)</t>
         </is>
       </c>
       <c r="N9" s="5" t="inlineStr">
@@ -1411,27 +1453,32 @@
       </c>
       <c r="O9" s="5" t="inlineStr">
         <is>
-          <t>Expo 2020 pavilions, Dubai towers, Ayedh Hussein Bin Dejem Real Estate</t>
+          <t>Not published</t>
         </is>
       </c>
       <c r="P9" s="5" t="inlineStr">
         <is>
-          <t>Dubai IFM with large cleaning and housekeeping workforce</t>
+          <t>Emirati-owned IFM competitor in Abu Dhabi</t>
         </is>
       </c>
       <c r="Q9" s="5" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>No government or state shareholder found in public sources</t>
         </is>
       </c>
       <c r="R9" s="5" t="inlineStr">
         <is>
-          <t>gulfnews.com (House Keeping deal); khaleejtimes.com; simplywall.st (UPP ownership)</t>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="S9" s="5" t="inlineStr">
+        <is>
+          <t>village.ai (AJAD FM); bayut.com (FM companies Abu Dhabi)</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:R9"/>
+  <autoFilter ref="A1:S9"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -1442,7 +1489,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R7"/>
+  <dimension ref="A1:S7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="4" customWidth="1" min="1" max="1"/>
@@ -1461,8 +1508,9 @@
     <col width="22" customWidth="1" min="14" max="14"/>
     <col width="30" customWidth="1" min="15" max="15"/>
     <col width="34" customWidth="1" min="16" max="16"/>
-    <col width="12" customWidth="1" min="17" max="17"/>
-    <col width="46" customWidth="1" min="18" max="18"/>
+    <col width="28" customWidth="1" min="17" max="17"/>
+    <col width="12" customWidth="1" min="18" max="18"/>
+    <col width="46" customWidth="1" min="19" max="19"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1548,10 +1596,15 @@
       </c>
       <c r="Q1" s="4" t="inlineStr">
         <is>
+          <t>Government ownership check</t>
+        </is>
+      </c>
+      <c r="R1" s="4" t="inlineStr">
+        <is>
           <t>Data confidence</t>
         </is>
       </c>
-      <c r="R1" s="4" t="inlineStr">
+      <c r="S1" s="4" t="inlineStr">
         <is>
           <t>Main sources</t>
         </is>
@@ -1563,32 +1616,32 @@
       </c>
       <c r="B2" s="7" t="inlineStr">
         <is>
-          <t>G4S Secure Solutions UAE</t>
+          <t>First Security Group (FSG)</t>
         </is>
       </c>
       <c r="C2" s="5" t="inlineStr">
         <is>
-          <t>Manned guarding, event security, cash services, electronic security, risk consulting</t>
+          <t>Manned guarding, security &amp; H&amp;S training (FSG Training Centre), investigations, due diligence</t>
         </is>
       </c>
       <c r="D2" s="5" t="inlineStr">
         <is>
-          <t>Allied Universal (USA, private; backed by Warburg Pincus and Canada's CDPQ). UAE local shareholding not published</t>
+          <t>Private; founded by 10 retired Dubai Police major generals. CEO Ret. Maj. Gen. Abdul Aziz Al Bannai</t>
         </is>
       </c>
       <c r="E2" s="5" t="inlineStr">
         <is>
-          <t>American (parent)</t>
+          <t>Emirati</t>
         </is>
       </c>
       <c r="F2" s="5" t="inlineStr">
         <is>
-          <t>Private (foreign multinational)</t>
+          <t>Private (100% local)</t>
         </is>
       </c>
       <c r="G2" s="5" t="inlineStr">
         <is>
-          <t>Operating in UAE for decades (G4S acquired 2021 by Allied Universal)</t>
+          <t>2004 (start-up capital AED 20M)</t>
         </is>
       </c>
       <c r="H2" s="5" t="inlineStr">
@@ -1598,52 +1651,57 @@
       </c>
       <c r="I2" s="5" t="inlineStr">
         <is>
-          <t>UAE (5 branches), wider region approx. 30,000 staff</t>
+          <t>UAE</t>
         </is>
       </c>
       <c r="J2" s="5" t="inlineStr">
         <is>
-          <t>9,000 (2021 report) to 12,000+ (G4S case study)</t>
+          <t>1,001 to 5,000 (GulfTalent/Naukri)</t>
         </is>
       </c>
       <c r="K2" s="5" t="inlineStr">
         <is>
-          <t>6,000+ SIRA/ASSD certified guards; 35 nationalities</t>
+          <t>Dubai Police-registered training centre</t>
         </is>
       </c>
       <c r="L2" s="5" t="inlineStr">
         <is>
-          <t>Not published for UAE</t>
+          <t>Not published</t>
         </is>
       </c>
       <c r="M2" s="5" t="inlineStr">
         <is>
-          <t>approx. AED 648M to 1,200M</t>
+          <t>approx. AED 72M to 500M</t>
         </is>
       </c>
       <c r="N2" s="5" t="inlineStr">
         <is>
-          <t>SIRA (Dubai), ASSD (Abu Dhabi)</t>
+          <t>SIRA; training registered with Dubai Police and Dubai Ambulance</t>
         </is>
       </c>
       <c r="O2" s="5" t="inlineStr">
         <is>
-          <t>Real estate developers, government-related venues, events</t>
+          <t>Corporate and government-related clients</t>
         </is>
       </c>
       <c r="P2" s="5" t="inlineStr">
         <is>
-          <t>Largest private guarding competitor for MEBS security division</t>
+          <t>Emirati-owned Dubai guarding firm, direct overlap with MEBS's origin business</t>
         </is>
       </c>
       <c r="Q2" s="5" t="inlineStr">
         <is>
+          <t>Private, 100% local. Founders are retired Dubai Police officers investing as private individuals; no government shareholder found</t>
+        </is>
+      </c>
+      <c r="R2" s="5" t="inlineStr">
+        <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="R2" s="5" t="inlineStr">
-        <is>
-          <t>g4s.com (UAE case study); securitymagazine.com (Allied deal); propertyfinder.ae</t>
+      <c r="S2" s="5" t="inlineStr">
+        <is>
+          <t>gulfnews.com (ex-police officers launch FSG; 'We know the meaning of security'); gulftalent.com</t>
         </is>
       </c>
     </row>
@@ -1653,32 +1711,32 @@
       </c>
       <c r="B3" s="7" t="inlineStr">
         <is>
-          <t>First Security Group (FSG)</t>
+          <t>Securitas UAE LLC</t>
         </is>
       </c>
       <c r="C3" s="5" t="inlineStr">
         <is>
-          <t>Manned guarding, security &amp; H&amp;S training (FSG Training Centre), investigations, due diligence</t>
+          <t>Specialised guarding, mobile patrol, security receptionists, electronic security, monitoring</t>
         </is>
       </c>
       <c r="D3" s="5" t="inlineStr">
         <is>
-          <t>Private; founded by 10 retired Dubai Police major generals. CEO Ret. Maj. Gen. Abdul Aziz Al Bannai</t>
+          <t>Securitas AB (Sweden; Nasdaq Stockholm listed)</t>
         </is>
       </c>
       <c r="E3" s="5" t="inlineStr">
         <is>
-          <t>Emirati</t>
+          <t>Swedish (parent)</t>
         </is>
       </c>
       <c r="F3" s="5" t="inlineStr">
         <is>
-          <t>Private (100% local)</t>
+          <t>Private (listed multinational)</t>
         </is>
       </c>
       <c r="G3" s="5" t="inlineStr">
         <is>
-          <t>2004 (start-up capital AED 20M)</t>
+          <t>2009 (UAE)</t>
         </is>
       </c>
       <c r="H3" s="5" t="inlineStr">
@@ -1693,47 +1751,52 @@
       </c>
       <c r="J3" s="5" t="inlineStr">
         <is>
-          <t>1,001 to 5,000 (GulfTalent/Naukri)</t>
+          <t>1,400+ (company); 201 to 1,000 (directories)</t>
         </is>
       </c>
       <c r="K3" s="5" t="inlineStr">
         <is>
-          <t>Dubai Police-registered training centre</t>
+          <t>400+ clients; 37% growth in 2014</t>
         </is>
       </c>
       <c r="L3" s="5" t="inlineStr">
         <is>
-          <t>Not published</t>
+          <t>Not published for UAE</t>
         </is>
       </c>
       <c r="M3" s="5" t="inlineStr">
         <is>
-          <t>approx. AED 72M to 500M</t>
+          <t>approx. AED 72M to 140M</t>
         </is>
       </c>
       <c r="N3" s="5" t="inlineStr">
         <is>
-          <t>SIRA; training registered with Dubai Police and Dubai Ambulance</t>
+          <t>SIRA</t>
         </is>
       </c>
       <c r="O3" s="5" t="inlineStr">
         <is>
-          <t>Corporate and government-related clients</t>
+          <t>Corporate offices, community sponsorship (Dubai Exiles RFC)</t>
         </is>
       </c>
       <c r="P3" s="5" t="inlineStr">
         <is>
-          <t>Emirati-owned Dubai guarding firm, direct overlap with MEBS's origin business</t>
+          <t>Competes on premium corporate guarding in Dubai</t>
         </is>
       </c>
       <c r="Q3" s="5" t="inlineStr">
         <is>
+          <t>Parent listed in Stockholm; main shareholders are private Swedish investment companies. No state owner</t>
+        </is>
+      </c>
+      <c r="R3" s="5" t="inlineStr">
+        <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="R3" s="5" t="inlineStr">
-        <is>
-          <t>gulfnews.com (ex-police officers launch FSG; 'We know the meaning of security'); gulftalent.com</t>
+      <c r="S3" s="5" t="inlineStr">
+        <is>
+          <t>tradearabia.com (37% growth 2014); zawya.com; dubaiexiles.com</t>
         </is>
       </c>
     </row>
@@ -1743,37 +1806,37 @@
       </c>
       <c r="B4" s="7" t="inlineStr">
         <is>
-          <t>Securitas UAE LLC</t>
+          <t>Magnum Security</t>
         </is>
       </c>
       <c r="C4" s="5" t="inlineStr">
         <is>
-          <t>Specialised guarding, mobile patrol, security receptionists, electronic security, monitoring</t>
+          <t>Security guards, consulting, VIP/close protection, security chauffeurs, CCTV monitoring</t>
         </is>
       </c>
       <c r="D4" s="5" t="inlineStr">
         <is>
-          <t>Securitas AB (Sweden; Nasdaq Stockholm listed)</t>
+          <t>Private. Managing Director Jimmy Singh (owner not published)</t>
         </is>
       </c>
       <c r="E4" s="5" t="inlineStr">
         <is>
-          <t>Swedish (parent)</t>
+          <t>Not published</t>
         </is>
       </c>
       <c r="F4" s="5" t="inlineStr">
         <is>
-          <t>Private (listed multinational)</t>
+          <t>Private</t>
         </is>
       </c>
       <c r="G4" s="5" t="inlineStr">
         <is>
-          <t>2009 (UAE)</t>
+          <t>2003</t>
         </is>
       </c>
       <c r="H4" s="5" t="inlineStr">
         <is>
-          <t>Dubai</t>
+          <t>Dubai (new facility planned in Jebel Ali)</t>
         </is>
       </c>
       <c r="I4" s="5" t="inlineStr">
@@ -1783,47 +1846,52 @@
       </c>
       <c r="J4" s="5" t="inlineStr">
         <is>
-          <t>1,400+ (company); 201 to 1,000 (directories)</t>
+          <t>1,000+ (company); 501 to 1,000 (ZoomInfo)</t>
         </is>
       </c>
       <c r="K4" s="5" t="inlineStr">
         <is>
-          <t>400+ clients; 37% growth in 2014</t>
+          <t>SIRA and SGS ISO 9001:2015 certified</t>
         </is>
       </c>
       <c r="L4" s="5" t="inlineStr">
         <is>
-          <t>Not published for UAE</t>
+          <t>Approx. US$44.5M (ZoomInfo estimate, unverified)</t>
         </is>
       </c>
       <c r="M4" s="5" t="inlineStr">
         <is>
-          <t>approx. AED 72M to 140M</t>
+          <t>approx. AED 36M to 100M</t>
         </is>
       </c>
       <c r="N4" s="5" t="inlineStr">
         <is>
-          <t>SIRA</t>
+          <t>SIRA, ISO 9001:2015</t>
         </is>
       </c>
       <c r="O4" s="5" t="inlineStr">
         <is>
-          <t>Corporate offices, community sponsorship (Dubai Exiles RFC)</t>
+          <t>Residential and commercial buildings</t>
         </is>
       </c>
       <c r="P4" s="5" t="inlineStr">
         <is>
-          <t>Competes on premium corporate guarding in Dubai</t>
+          <t>Similar-size Dubai guarding firm, direct price competitor</t>
         </is>
       </c>
       <c r="Q4" s="5" t="inlineStr">
         <is>
+          <t>No government or state shareholder found in public sources</t>
+        </is>
+      </c>
+      <c r="R4" s="5" t="inlineStr">
+        <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="R4" s="5" t="inlineStr">
-        <is>
-          <t>tradearabia.com (37% growth 2014); zawya.com; dubaiexiles.com</t>
+      <c r="S4" s="5" t="inlineStr">
+        <is>
+          <t>khaleejtimes.com ('Security that matters', 'Think safety with Magnum'); magnumsecurity.ae; zoominfo.com</t>
         </is>
       </c>
     </row>
@@ -1833,87 +1901,92 @@
       </c>
       <c r="B5" s="7" t="inlineStr">
         <is>
-          <t>Magnum Security</t>
+          <t>Landmark Security Services</t>
         </is>
       </c>
       <c r="C5" s="5" t="inlineStr">
         <is>
-          <t>Security guards, consulting, VIP/close protection, security chauffeurs, CCTV monitoring</t>
+          <t>Manned guarding for residential and corporate clients</t>
         </is>
       </c>
       <c r="D5" s="5" t="inlineStr">
         <is>
-          <t>Private. Managing Director Jimmy Singh (owner not published)</t>
+          <t>Private. MD Rashid Almoosa, founder Salim Nahfaoui (third-party data, unverified)</t>
         </is>
       </c>
       <c r="E5" s="5" t="inlineStr">
         <is>
+          <t>Not confirmed</t>
+        </is>
+      </c>
+      <c r="F5" s="5" t="inlineStr">
+        <is>
+          <t>Private</t>
+        </is>
+      </c>
+      <c r="G5" s="5" t="inlineStr">
+        <is>
+          <t>2004</t>
+        </is>
+      </c>
+      <c r="H5" s="5" t="inlineStr">
+        <is>
+          <t>Al Sufouh, Dubai</t>
+        </is>
+      </c>
+      <c r="I5" s="5" t="inlineStr">
+        <is>
+          <t>UAE</t>
+        </is>
+      </c>
+      <c r="J5" s="5" t="inlineStr">
+        <is>
+          <t>800+ (company/ZoomInfo)</t>
+        </is>
+      </c>
+      <c r="K5" s="5" t="inlineStr">
+        <is>
+          <t>SIRA certified</t>
+        </is>
+      </c>
+      <c r="L5" s="5" t="inlineStr">
+        <is>
           <t>Not published</t>
         </is>
       </c>
-      <c r="F5" s="5" t="inlineStr">
-        <is>
-          <t>Private</t>
-        </is>
-      </c>
-      <c r="G5" s="5" t="inlineStr">
-        <is>
-          <t>2003</t>
-        </is>
-      </c>
-      <c r="H5" s="5" t="inlineStr">
-        <is>
-          <t>Dubai (new facility planned in Jebel Ali)</t>
-        </is>
-      </c>
-      <c r="I5" s="5" t="inlineStr">
-        <is>
-          <t>UAE</t>
-        </is>
-      </c>
-      <c r="J5" s="5" t="inlineStr">
-        <is>
-          <t>1,000+ (company); 501 to 1,000 (ZoomInfo)</t>
-        </is>
-      </c>
-      <c r="K5" s="5" t="inlineStr">
-        <is>
-          <t>SIRA and SGS ISO 9001:2015 certified</t>
-        </is>
-      </c>
-      <c r="L5" s="5" t="inlineStr">
-        <is>
-          <t>Approx. US$44.5M (ZoomInfo estimate, unverified)</t>
-        </is>
-      </c>
       <c r="M5" s="5" t="inlineStr">
         <is>
-          <t>approx. AED 36M to 100M</t>
+          <t>approx. AED 58M to 100M</t>
         </is>
       </c>
       <c r="N5" s="5" t="inlineStr">
         <is>
-          <t>SIRA, ISO 9001:2015</t>
+          <t>SIRA</t>
         </is>
       </c>
       <c r="O5" s="5" t="inlineStr">
         <is>
-          <t>Residential and commercial buildings</t>
+          <t>Residential communities, corporate</t>
         </is>
       </c>
       <c r="P5" s="5" t="inlineStr">
         <is>
-          <t>Similar-size Dubai guarding firm, direct price competitor</t>
+          <t>Size peer of MEBS in Dubai guarding</t>
         </is>
       </c>
       <c r="Q5" s="5" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>No government or state shareholder found in public sources</t>
         </is>
       </c>
       <c r="R5" s="5" t="inlineStr">
         <is>
-          <t>khaleejtimes.com ('Security that matters', 'Think safety with Magnum'); magnumsecurity.ae; zoominfo.com</t>
+          <t>Low to medium</t>
+        </is>
+      </c>
+      <c r="S5" s="5" t="inlineStr">
+        <is>
+          <t>landmarksecurity.ae; dubizzle.com (security companies); zoominfo.com; prospeo.io</t>
         </is>
       </c>
     </row>
@@ -1923,17 +1996,17 @@
       </c>
       <c r="B6" s="7" t="inlineStr">
         <is>
-          <t>Landmark Security Services</t>
+          <t>Guardforce Security Services UAE</t>
         </is>
       </c>
       <c r="C6" s="5" t="inlineStr">
         <is>
-          <t>Manned guarding for residential and corporate clients</t>
+          <t>SIRA-licensed manned guarding for retail, education, hospitality, commercial and industrial</t>
         </is>
       </c>
       <c r="D6" s="5" t="inlineStr">
         <is>
-          <t>Private. MD Rashid Almoosa, founder Salim Nahfaoui (third-party data, unverified)</t>
+          <t>Private. CEO Mick Iqbal (Indeed listing). Ultimate owner not published</t>
         </is>
       </c>
       <c r="E6" s="5" t="inlineStr">
@@ -1948,12 +2021,12 @@
       </c>
       <c r="G6" s="5" t="inlineStr">
         <is>
-          <t>2004</t>
+          <t>April 2007 (Dubai office)</t>
         </is>
       </c>
       <c r="H6" s="5" t="inlineStr">
         <is>
-          <t>Al Sufouh, Dubai</t>
+          <t>Jumeirah Village Circle, Dubai</t>
         </is>
       </c>
       <c r="I6" s="5" t="inlineStr">
@@ -1963,12 +2036,12 @@
       </c>
       <c r="J6" s="5" t="inlineStr">
         <is>
-          <t>800+ (company/ZoomInfo)</t>
+          <t>201 to 500 (aggregator)</t>
         </is>
       </c>
       <c r="K6" s="5" t="inlineStr">
         <is>
-          <t>SIRA certified</t>
+          <t>Multi-sector guarding</t>
         </is>
       </c>
       <c r="L6" s="5" t="inlineStr">
@@ -1978,7 +2051,7 @@
       </c>
       <c r="M6" s="5" t="inlineStr">
         <is>
-          <t>approx. AED 58M to 100M</t>
+          <t>approx. AED 14M to 50M</t>
         </is>
       </c>
       <c r="N6" s="5" t="inlineStr">
@@ -1988,22 +2061,27 @@
       </c>
       <c r="O6" s="5" t="inlineStr">
         <is>
-          <t>Residential communities, corporate</t>
+          <t>Retail, schools, hotels</t>
         </is>
       </c>
       <c r="P6" s="5" t="inlineStr">
         <is>
-          <t>Size peer of MEBS in Dubai guarding</t>
+          <t>Smaller Dubai guarding competitor in the same segments</t>
         </is>
       </c>
       <c r="Q6" s="5" t="inlineStr">
         <is>
-          <t>Low to medium</t>
+          <t>No government or state shareholder found in public sources</t>
         </is>
       </c>
       <c r="R6" s="5" t="inlineStr">
         <is>
-          <t>landmarksecurity.ae; dubizzle.com (security companies); zoominfo.com; prospeo.io</t>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="S6" s="5" t="inlineStr">
+        <is>
+          <t>guardforce.ae; ae.indeed.com; prospeo.io</t>
         </is>
       </c>
     </row>
@@ -2013,37 +2091,37 @@
       </c>
       <c r="B7" s="7" t="inlineStr">
         <is>
-          <t>Guardforce Security Services UAE</t>
+          <t>Al Manal Security LLC</t>
         </is>
       </c>
       <c r="C7" s="5" t="inlineStr">
         <is>
-          <t>SIRA-licensed manned guarding for retail, education, hospitality, commercial and industrial</t>
+          <t>Private security guarding and investigations, community-focused contracts</t>
         </is>
       </c>
       <c r="D7" s="5" t="inlineStr">
         <is>
-          <t>Private. CEO Mick Iqbal (Indeed listing). Ultimate owner not published</t>
+          <t>Juma Ahmad Majid Al Ghurair and Marwan Ahmad Majid Al Ghurair (per business directory, unverified)</t>
         </is>
       </c>
       <c r="E7" s="5" t="inlineStr">
         <is>
-          <t>Not confirmed</t>
+          <t>Emirati</t>
         </is>
       </c>
       <c r="F7" s="5" t="inlineStr">
         <is>
-          <t>Private</t>
+          <t>Private family</t>
         </is>
       </c>
       <c r="G7" s="5" t="inlineStr">
         <is>
-          <t>April 2007 (Dubai office)</t>
+          <t>2005</t>
         </is>
       </c>
       <c r="H7" s="5" t="inlineStr">
         <is>
-          <t>Jumeirah Village Circle, Dubai</t>
+          <t>Dubai Silicon Oasis, Dubai</t>
         </is>
       </c>
       <c r="I7" s="5" t="inlineStr">
@@ -2053,12 +2131,12 @@
       </c>
       <c r="J7" s="5" t="inlineStr">
         <is>
-          <t>201 to 500 (aggregator)</t>
+          <t>80+ (directory)</t>
         </is>
       </c>
       <c r="K7" s="5" t="inlineStr">
         <is>
-          <t>Multi-sector guarding</t>
+          <t>Small and community contracts</t>
         </is>
       </c>
       <c r="L7" s="5" t="inlineStr">
@@ -2068,7 +2146,7 @@
       </c>
       <c r="M7" s="5" t="inlineStr">
         <is>
-          <t>approx. AED 14M to 50M</t>
+          <t>approx. AED 6M to 15M</t>
         </is>
       </c>
       <c r="N7" s="5" t="inlineStr">
@@ -2078,27 +2156,32 @@
       </c>
       <c r="O7" s="5" t="inlineStr">
         <is>
-          <t>Retail, schools, hotels</t>
+          <t>Residential communities</t>
         </is>
       </c>
       <c r="P7" s="5" t="inlineStr">
         <is>
-          <t>Smaller Dubai guarding competitor in the same segments</t>
+          <t>Emirati family-owned Dubai guarding firm</t>
         </is>
       </c>
       <c r="Q7" s="5" t="inlineStr">
         <is>
+          <t>No government or state shareholder found in public sources</t>
+        </is>
+      </c>
+      <c r="R7" s="5" t="inlineStr">
+        <is>
           <t>Low</t>
         </is>
       </c>
-      <c r="R7" s="5" t="inlineStr">
-        <is>
-          <t>guardforce.ae; ae.indeed.com; prospeo.io</t>
+      <c r="S7" s="5" t="inlineStr">
+        <is>
+          <t>village.ai (Al Manal Security); contactout.com; propertyfinder.ae</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:R7"/>
+  <autoFilter ref="A1:S7"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -2109,7 +2192,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R7"/>
+  <dimension ref="A1:S7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="4" customWidth="1" min="1" max="1"/>
@@ -2128,8 +2211,9 @@
     <col width="22" customWidth="1" min="14" max="14"/>
     <col width="30" customWidth="1" min="15" max="15"/>
     <col width="34" customWidth="1" min="16" max="16"/>
-    <col width="12" customWidth="1" min="17" max="17"/>
-    <col width="46" customWidth="1" min="18" max="18"/>
+    <col width="28" customWidth="1" min="17" max="17"/>
+    <col width="12" customWidth="1" min="18" max="18"/>
+    <col width="46" customWidth="1" min="19" max="19"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -2215,10 +2299,15 @@
       </c>
       <c r="Q1" s="4" t="inlineStr">
         <is>
+          <t>Government ownership check</t>
+        </is>
+      </c>
+      <c r="R1" s="4" t="inlineStr">
+        <is>
           <t>Data confidence</t>
         </is>
       </c>
-      <c r="R1" s="4" t="inlineStr">
+      <c r="S1" s="4" t="inlineStr">
         <is>
           <t>Main sources</t>
         </is>
@@ -2305,10 +2394,15 @@
       </c>
       <c r="Q2" s="5" t="inlineStr">
         <is>
+          <t>No government or state shareholder found in public sources</t>
+        </is>
+      </c>
+      <c r="R2" s="5" t="inlineStr">
+        <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="R2" s="5" t="inlineStr">
+      <c r="S2" s="5" t="inlineStr">
         <is>
           <t>gulftalent.com (Cleanco); mefma.org (Cleanco Group); zawya.com (Guinness record); sustainabilitymenews.com</t>
         </is>
@@ -2395,10 +2489,15 @@
       </c>
       <c r="Q3" s="5" t="inlineStr">
         <is>
+          <t>Owned by the Klüh family company (Germany). No state owner</t>
+        </is>
+      </c>
+      <c r="R3" s="5" t="inlineStr">
+        <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="R3" s="5" t="inlineStr">
+      <c r="S3" s="5" t="inlineStr">
         <is>
           <t>klueh.de (Burj Khalifa extension 2020; Cleaning Company of the Year 2018; UAE page)</t>
         </is>
@@ -2485,10 +2584,15 @@
       </c>
       <c r="Q4" s="5" t="inlineStr">
         <is>
+          <t>Owned by Dussmann Group (German private family/foundation). No state owner</t>
+        </is>
+      </c>
+      <c r="R4" s="5" t="inlineStr">
+        <is>
           <t>Low to medium</t>
         </is>
       </c>
-      <c r="R4" s="5" t="inlineStr">
+      <c r="S4" s="5" t="inlineStr">
         <is>
           <t>dussmann.ae; reveliolabs.com; mefma.org</t>
         </is>
@@ -2575,10 +2679,15 @@
       </c>
       <c r="Q5" s="5" t="inlineStr">
         <is>
+          <t>No government or state shareholder found in public sources</t>
+        </is>
+      </c>
+      <c r="R5" s="5" t="inlineStr">
+        <is>
           <t>Low</t>
         </is>
       </c>
-      <c r="R5" s="5" t="inlineStr">
+      <c r="S5" s="5" t="inlineStr">
         <is>
           <t>naukrigulf.com; zoominfo.com; mefma.org (White Spot FM)</t>
         </is>
@@ -2665,10 +2774,15 @@
       </c>
       <c r="Q6" s="5" t="inlineStr">
         <is>
+          <t>No government or state shareholder found in public sources</t>
+        </is>
+      </c>
+      <c r="R6" s="5" t="inlineStr">
+        <is>
           <t>Low to medium</t>
         </is>
       </c>
-      <c r="R6" s="5" t="inlineStr">
+      <c r="S6" s="5" t="inlineStr">
         <is>
           <t>bitscale.ai; wamda.com; zoominfo.com; prospeo.io</t>
         </is>
@@ -2755,17 +2869,22 @@
       </c>
       <c r="Q7" s="5" t="inlineStr">
         <is>
+          <t>No government or state shareholder found in public sources</t>
+        </is>
+      </c>
+      <c r="R7" s="5" t="inlineStr">
+        <is>
           <t>Low</t>
         </is>
       </c>
-      <c r="R7" s="5" t="inlineStr">
+      <c r="S7" s="5" t="inlineStr">
         <is>
           <t>albwardy.com (Total Care Cleaning Services page)</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:R7"/>
+  <autoFilter ref="A1:S7"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -2914,7 +3033,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B10"/>
+  <dimension ref="A1:B16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -3041,6 +3160,78 @@
         </is>
       </c>
     </row>
+    <row r="11">
+      <c r="A11" s="11" t="inlineStr">
+        <is>
+          <t>Enova by Veolia</t>
+        </is>
+      </c>
+      <c r="B11" s="5" t="inlineStr">
+        <is>
+          <t>JV partner Veolia has the French state-owned Caisse des Dépôts as a shareholder (approx. 4.6%)</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="11" t="inlineStr">
+        <is>
+          <t>G4S UAE</t>
+        </is>
+      </c>
+      <c r="B12" s="5" t="inlineStr">
+        <is>
+          <t>Parent Allied Universal is co-owned by CDPQ, the Quebec government's pension fund</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="11" t="inlineStr">
+        <is>
+          <t>ServeU</t>
+        </is>
+      </c>
+      <c r="B13" s="5" t="inlineStr">
+        <is>
+          <t>Parent Union Properties has had Emirates NBD (government-owned bank) as a major shareholder</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="11" t="inlineStr">
+        <is>
+          <t>Dulsco Group</t>
+        </is>
+      </c>
+      <c r="B14" s="5" t="inlineStr">
+        <is>
+          <t>Shareholder is a member of the Dubai ruling family; excluded to stay on the safe side</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="11" t="inlineStr">
+        <is>
+          <t>Mace Macro Technical Services</t>
+        </is>
+      </c>
+      <c r="B15" s="5" t="inlineStr">
+        <is>
+          <t>Acquired by Khidmah (Aldar group) in 2022</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="11" t="inlineStr">
+        <is>
+          <t>Al Tanmyah Services</t>
+        </is>
+      </c>
+      <c r="B16" s="5" t="inlineStr">
+        <is>
+          <t>Subsidiary of Dubai Islamic Bank (government shareholding)</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Expand to 20 companies per category and apply MEBS branding to page
Add 12 FM, 14 security and 14 cleaning companies (extra_data.py), all
without government owners; 11 more government-linked firms added to
the exclusions list. Restyle the HTML page with MEBS brand colours,
blue gradient hero, rounded cards and a slot for the MEBS logo file
(mebs-logo.png next to the page, text wordmark fallback).

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01QTLqykBaXLnYN7UB8pKnAZ
</commit_message>
<xml_diff>
--- a/research/mebs-competitors/MEBS_Competitors_UAE.xlsx
+++ b/research/mebs-competitors/MEBS_Competitors_UAE.xlsx
@@ -15,9 +15,9 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Excluded (gov-linked)" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'FM Companies'!$A$1:$S$9</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Security Only'!$A$1:$S$7</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Cleaning Only'!$A$1:$S$7</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'FM Companies'!$A$1:$S$21</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Security Only'!$A$1:$S$21</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Cleaning Only'!$A$1:$S$21</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -504,7 +504,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>MEBS Facility Services: 20 private-sector competitors (UAE)</t>
+          <t>MEBS Facility Services: 60 private-sector competitors (UAE), 20 per category</t>
         </is>
       </c>
     </row>
@@ -528,7 +528,7 @@
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>1. FM Companies (8)  2. Security Only (6)  3. Cleaning Only (6)  4. MEBS benchmark  5. Excluded (gov-linked)
+          <t>1. FM Companies (20)  2. Security Only (20)  3. Cleaning Only (20)  4. MEBS benchmark  5. Excluded (gov-linked)
 Separate files are also provided per category.</t>
         </is>
       </c>
@@ -596,7 +596,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:S9"/>
+  <dimension ref="A1:S21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="4" customWidth="1" min="1" max="1"/>
@@ -1477,8 +1477,1148 @@
         </is>
       </c>
     </row>
+    <row r="10">
+      <c r="A10" s="5" t="n">
+        <v>9</v>
+      </c>
+      <c r="B10" s="6" t="inlineStr">
+        <is>
+          <t>Khansaheb Facilities Management</t>
+        </is>
+      </c>
+      <c r="C10" s="5" t="inlineStr">
+        <is>
+          <t>Integrated FM: MEP, civil maintenance, soft services; grew out of Khansaheb's construction business</t>
+        </is>
+      </c>
+      <c r="D10" s="5" t="inlineStr">
+        <is>
+          <t>Khansaheb Investment LLC (Khansaheb family). Chairman Tariq Hussain Khansaheb. Bought back Interserve's stakes in group companies</t>
+        </is>
+      </c>
+      <c r="E10" s="5" t="inlineStr">
+        <is>
+          <t>Emirati</t>
+        </is>
+      </c>
+      <c r="F10" s="5" t="inlineStr">
+        <is>
+          <t>Private family group</t>
+        </is>
+      </c>
+      <c r="G10" s="5" t="inlineStr">
+        <is>
+          <t>Group 1935; FM company (Khansaheb FMS LLC) 2020</t>
+        </is>
+      </c>
+      <c r="H10" s="5" t="inlineStr">
+        <is>
+          <t>Dubai</t>
+        </is>
+      </c>
+      <c r="I10" s="5" t="inlineStr">
+        <is>
+          <t>UAE</t>
+        </is>
+      </c>
+      <c r="J10" s="5" t="inlineStr">
+        <is>
+          <t>501 to 1,000 (aggregator); group 5,000+</t>
+        </is>
+      </c>
+      <c r="K10" s="5" t="inlineStr">
+        <is>
+          <t>Backed by a 90-year-old contracting group</t>
+        </is>
+      </c>
+      <c r="L10" s="5" t="inlineStr">
+        <is>
+          <t>Not published</t>
+        </is>
+      </c>
+      <c r="M10" s="5" t="inlineStr">
+        <is>
+          <t>approx. AED 38M to 110M</t>
+        </is>
+      </c>
+      <c r="N10" s="5" t="inlineStr">
+        <is>
+          <t>Not published</t>
+        </is>
+      </c>
+      <c r="O10" s="5" t="inlineStr">
+        <is>
+          <t>Commercial and community portfolios</t>
+        </is>
+      </c>
+      <c r="P10" s="5" t="inlineStr">
+        <is>
+          <t>Emirati family-owned IFM in Dubai competing for MEP and soft-services contracts</t>
+        </is>
+      </c>
+      <c r="Q10" s="5" t="inlineStr">
+        <is>
+          <t>No government or state shareholder found in public sources</t>
+        </is>
+      </c>
+      <c r="R10" s="5" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="S10" s="5" t="inlineStr">
+        <is>
+          <t>forbesmiddleeast.com (Khansaheb Group); zawya.com (buyback from Interserve); cm-today.com</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="5" t="n">
+        <v>10</v>
+      </c>
+      <c r="B11" s="6" t="inlineStr">
+        <is>
+          <t>ADEEB Group</t>
+        </is>
+      </c>
+      <c r="C11" s="5" t="inlineStr">
+        <is>
+          <t>Integrated FM, MEP contracting, HVAC operation and maintenance</t>
+        </is>
+      </c>
+      <c r="D11" s="5" t="inlineStr">
+        <is>
+          <t>Sultan Bin Rashed (SBR) Group, owned by Sultan Bin Rashed Al Dhaheri</t>
+        </is>
+      </c>
+      <c r="E11" s="5" t="inlineStr">
+        <is>
+          <t>Emirati</t>
+        </is>
+      </c>
+      <c r="F11" s="5" t="inlineStr">
+        <is>
+          <t>Private family group</t>
+        </is>
+      </c>
+      <c r="G11" s="5" t="inlineStr">
+        <is>
+          <t>1994</t>
+        </is>
+      </c>
+      <c r="H11" s="5" t="inlineStr">
+        <is>
+          <t>Sama Tower, Madinat Zayed, Abu Dhabi</t>
+        </is>
+      </c>
+      <c r="I11" s="5" t="inlineStr">
+        <is>
+          <t>Abu Dhabi, Dubai, Al Ain, Ajman, Mussafah</t>
+        </is>
+      </c>
+      <c r="J11" s="5" t="inlineStr">
+        <is>
+          <t>501 to 1,000 (Naukri, ZoomInfo)</t>
+        </is>
+      </c>
+      <c r="K11" s="5" t="inlineStr">
+        <is>
+          <t>Branches in Dubai, Al Ain, Ajman and Mussafah</t>
+        </is>
+      </c>
+      <c r="L11" s="5" t="inlineStr">
+        <is>
+          <t>Not published</t>
+        </is>
+      </c>
+      <c r="M11" s="5" t="inlineStr">
+        <is>
+          <t>approx. AED 38M to 110M</t>
+        </is>
+      </c>
+      <c r="N11" s="5" t="inlineStr">
+        <is>
+          <t>ISO 9001, 14001, 45001, 41001, 50001</t>
+        </is>
+      </c>
+      <c r="O11" s="5" t="inlineStr">
+        <is>
+          <t>Commercial and industrial clients in Abu Dhabi</t>
+        </is>
+      </c>
+      <c r="P11" s="5" t="inlineStr">
+        <is>
+          <t>Emirati-owned IFM with strong Abu Dhabi base</t>
+        </is>
+      </c>
+      <c r="Q11" s="5" t="inlineStr">
+        <is>
+          <t>No government or state shareholder found in public sources</t>
+        </is>
+      </c>
+      <c r="R11" s="5" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="S11" s="5" t="inlineStr">
+        <is>
+          <t>mefma.org (Adeeb Group); bayut.com (Abu Dhabi FM list); naukrigulf.com</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="5" t="n">
+        <v>11</v>
+      </c>
+      <c r="B12" s="6" t="inlineStr">
+        <is>
+          <t>Latinem Facilities Management</t>
+        </is>
+      </c>
+      <c r="C12" s="5" t="inlineStr">
+        <is>
+          <t>Technology-driven integrated FM: MEP, soft services, helpdesk</t>
+        </is>
+      </c>
+      <c r="D12" s="5" t="inlineStr">
+        <is>
+          <t>Private. Owner not published</t>
+        </is>
+      </c>
+      <c r="E12" s="5" t="inlineStr">
+        <is>
+          <t>Not published</t>
+        </is>
+      </c>
+      <c r="F12" s="5" t="inlineStr">
+        <is>
+          <t>Private</t>
+        </is>
+      </c>
+      <c r="G12" s="5" t="inlineStr">
+        <is>
+          <t>2014</t>
+        </is>
+      </c>
+      <c r="H12" s="5" t="inlineStr">
+        <is>
+          <t>Sobha Hartland Greens, Nad Al Sheba, Dubai</t>
+        </is>
+      </c>
+      <c r="I12" s="5" t="inlineStr">
+        <is>
+          <t>UAE</t>
+        </is>
+      </c>
+      <c r="J12" s="5" t="inlineStr">
+        <is>
+          <t>90+ (directory)</t>
+        </is>
+      </c>
+      <c r="K12" s="5" t="inlineStr">
+        <is>
+          <t>Residential communities and towers</t>
+        </is>
+      </c>
+      <c r="L12" s="5" t="inlineStr">
+        <is>
+          <t>Not published</t>
+        </is>
+      </c>
+      <c r="M12" s="5" t="inlineStr">
+        <is>
+          <t>approx. AED 7M to 16M</t>
+        </is>
+      </c>
+      <c r="N12" s="5" t="inlineStr">
+        <is>
+          <t>Not published</t>
+        </is>
+      </c>
+      <c r="O12" s="5" t="inlineStr">
+        <is>
+          <t>Owners associations and residential communities</t>
+        </is>
+      </c>
+      <c r="P12" s="5" t="inlineStr">
+        <is>
+          <t>Dubai IFM competing for owners-association and community contracts</t>
+        </is>
+      </c>
+      <c r="Q12" s="5" t="inlineStr">
+        <is>
+          <t>No government or state shareholder found in public sources</t>
+        </is>
+      </c>
+      <c r="R12" s="5" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="S12" s="5" t="inlineStr">
+        <is>
+          <t>mefma.org (Latinem FM); village.ai; dubizzle.com (FM companies Dubai)</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="5" t="n">
+        <v>12</v>
+      </c>
+      <c r="B13" s="6" t="inlineStr">
+        <is>
+          <t>Living Stone Facilities Management LLC</t>
+        </is>
+      </c>
+      <c r="C13" s="5" t="inlineStr">
+        <is>
+          <t>Facility management with an industrial-sector focus</t>
+        </is>
+      </c>
+      <c r="D13" s="5" t="inlineStr">
+        <is>
+          <t>Private. Owner not published</t>
+        </is>
+      </c>
+      <c r="E13" s="5" t="inlineStr">
+        <is>
+          <t>Not published</t>
+        </is>
+      </c>
+      <c r="F13" s="5" t="inlineStr">
+        <is>
+          <t>Private</t>
+        </is>
+      </c>
+      <c r="G13" s="5" t="inlineStr">
+        <is>
+          <t>Not published</t>
+        </is>
+      </c>
+      <c r="H13" s="5" t="inlineStr">
+        <is>
+          <t>Abu Dhabi</t>
+        </is>
+      </c>
+      <c r="I13" s="5" t="inlineStr">
+        <is>
+          <t>UAE</t>
+        </is>
+      </c>
+      <c r="J13" s="5" t="inlineStr">
+        <is>
+          <t>Not published</t>
+        </is>
+      </c>
+      <c r="K13" s="5" t="inlineStr">
+        <is>
+          <t>Described as one of the larger FM firms in Abu Dhabi</t>
+        </is>
+      </c>
+      <c r="L13" s="5" t="inlineStr">
+        <is>
+          <t>Not published</t>
+        </is>
+      </c>
+      <c r="M13" s="5" t="inlineStr">
+        <is>
+          <t>Cannot estimate (headcount unknown)</t>
+        </is>
+      </c>
+      <c r="N13" s="5" t="inlineStr">
+        <is>
+          <t>Not published</t>
+        </is>
+      </c>
+      <c r="O13" s="5" t="inlineStr">
+        <is>
+          <t>Industrial clients</t>
+        </is>
+      </c>
+      <c r="P13" s="5" t="inlineStr">
+        <is>
+          <t>Abu Dhabi FM competitor in industrial sites</t>
+        </is>
+      </c>
+      <c r="Q13" s="5" t="inlineStr">
+        <is>
+          <t>No government or state shareholder found in public sources</t>
+        </is>
+      </c>
+      <c r="R13" s="5" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="S13" s="5" t="inlineStr">
+        <is>
+          <t>bayut.com (FM companies Abu Dhabi); ensun.io</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="5" t="n">
+        <v>13</v>
+      </c>
+      <c r="B14" s="6" t="inlineStr">
+        <is>
+          <t>Sodexo Middle East</t>
+        </is>
+      </c>
+      <c r="C14" s="5" t="inlineStr">
+        <is>
+          <t>Integrated FM: catering, reception, maintenance, cleaning, facilities and equipment management</t>
+        </is>
+      </c>
+      <c r="D14" s="5" t="inlineStr">
+        <is>
+          <t>Sodexo SA (France; listed, controlled by the Bellon family). Operates through joint ventures in Dubai and Abu Dhabi (Sodexo | Kelvin)</t>
+        </is>
+      </c>
+      <c r="E14" s="5" t="inlineStr">
+        <is>
+          <t>French (parent)</t>
+        </is>
+      </c>
+      <c r="F14" s="5" t="inlineStr">
+        <is>
+          <t>Private (listed multinational, family-controlled)</t>
+        </is>
+      </c>
+      <c r="G14" s="5" t="inlineStr">
+        <is>
+          <t>In UAE since 1974; Kelvin (Abu Dhabi) since 1984</t>
+        </is>
+      </c>
+      <c r="H14" s="5" t="inlineStr">
+        <is>
+          <t>Dubai Silicon Oasis, Dubai</t>
+        </is>
+      </c>
+      <c r="I14" s="5" t="inlineStr">
+        <is>
+          <t>UAE, Oman, Qatar</t>
+        </is>
+      </c>
+      <c r="J14" s="5" t="inlineStr">
+        <is>
+          <t>Not published for UAE</t>
+        </is>
+      </c>
+      <c r="K14" s="5" t="inlineStr">
+        <is>
+          <t>Global group; healthcare, education and corporate sites</t>
+        </is>
+      </c>
+      <c r="L14" s="5" t="inlineStr">
+        <is>
+          <t>Not published for UAE</t>
+        </is>
+      </c>
+      <c r="M14" s="5" t="inlineStr">
+        <is>
+          <t>Cannot estimate (headcount unknown)</t>
+        </is>
+      </c>
+      <c r="N14" s="5" t="inlineStr">
+        <is>
+          <t>Not published</t>
+        </is>
+      </c>
+      <c r="O14" s="5" t="inlineStr">
+        <is>
+          <t>Healthcare, education and corporate sites</t>
+        </is>
+      </c>
+      <c r="P14" s="5" t="inlineStr">
+        <is>
+          <t>Global soft-services and IFM player bidding for large corporate contracts</t>
+        </is>
+      </c>
+      <c r="Q14" s="5" t="inlineStr">
+        <is>
+          <t>Parent controlled by the Bellon family; no state owner found. Local JV partners not published, so verify</t>
+        </is>
+      </c>
+      <c r="R14" s="5" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="S14" s="5" t="inlineStr">
+        <is>
+          <t>middleeast.sodexo.com (Kelvin Catering Services); zawya.com (Sodexo healthcare release)</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="5" t="n">
+        <v>14</v>
+      </c>
+      <c r="B15" s="6" t="inlineStr">
+        <is>
+          <t>Kharafi National</t>
+        </is>
+      </c>
+      <c r="C15" s="5" t="inlineStr">
+        <is>
+          <t>Construction, operation &amp; maintenance and facilities management</t>
+        </is>
+      </c>
+      <c r="D15" s="5" t="inlineStr">
+        <is>
+          <t>M. A. Kharafi &amp; Sons Group (Kharafi family, Kuwait)</t>
+        </is>
+      </c>
+      <c r="E15" s="5" t="inlineStr">
+        <is>
+          <t>Kuwaiti</t>
+        </is>
+      </c>
+      <c r="F15" s="5" t="inlineStr">
+        <is>
+          <t>Private family group</t>
+        </is>
+      </c>
+      <c r="G15" s="5" t="inlineStr">
+        <is>
+          <t>UAE branch 1995 (Dubai), Abu Dhabi 1996</t>
+        </is>
+      </c>
+      <c r="H15" s="5" t="inlineStr">
+        <is>
+          <t>Kuwait (UAE offices in Dubai and Abu Dhabi)</t>
+        </is>
+      </c>
+      <c r="I15" s="5" t="inlineStr">
+        <is>
+          <t>UAE, Kuwait, Qatar, Bahrain, Egypt</t>
+        </is>
+      </c>
+      <c r="J15" s="5" t="inlineStr">
+        <is>
+          <t>5,150 to 25,000+ group-wide (sources conflict)</t>
+        </is>
+      </c>
+      <c r="K15" s="5" t="inlineStr">
+        <is>
+          <t>Large O&amp;M contractor for infrastructure and utilities</t>
+        </is>
+      </c>
+      <c r="L15" s="5" t="inlineStr">
+        <is>
+          <t>Not published</t>
+        </is>
+      </c>
+      <c r="M15" s="5" t="inlineStr">
+        <is>
+          <t>Cannot estimate (headcount unknown)</t>
+        </is>
+      </c>
+      <c r="N15" s="5" t="inlineStr">
+        <is>
+          <t>Not published</t>
+        </is>
+      </c>
+      <c r="O15" s="5" t="inlineStr">
+        <is>
+          <t>Infrastructure and utilities O&amp;M</t>
+        </is>
+      </c>
+      <c r="P15" s="5" t="inlineStr">
+        <is>
+          <t>Competes for large O&amp;M and FM contracts</t>
+        </is>
+      </c>
+      <c r="Q15" s="5" t="inlineStr">
+        <is>
+          <t>No government or state shareholder found in public sources</t>
+        </is>
+      </c>
+      <c r="R15" s="5" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="S15" s="5" t="inlineStr">
+        <is>
+          <t>meed.com (Kharafi National); highperformr.ai; aeconline.ae</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="5" t="n">
+        <v>15</v>
+      </c>
+      <c r="B16" s="6" t="inlineStr">
+        <is>
+          <t>AG Facilities Solutions (AGFS)</t>
+        </is>
+      </c>
+      <c r="C16" s="5" t="inlineStr">
+        <is>
+          <t>Total FM and contracting: MEP, cleaning, soft services</t>
+        </is>
+      </c>
+      <c r="D16" s="5" t="inlineStr">
+        <is>
+          <t>Al Ghurair Group (Al Ghurair Investment)</t>
+        </is>
+      </c>
+      <c r="E16" s="5" t="inlineStr">
+        <is>
+          <t>Emirati</t>
+        </is>
+      </c>
+      <c r="F16" s="5" t="inlineStr">
+        <is>
+          <t>Private family group</t>
+        </is>
+      </c>
+      <c r="G16" s="5" t="inlineStr">
+        <is>
+          <t>2003 to 2006 (sources conflict)</t>
+        </is>
+      </c>
+      <c r="H16" s="5" t="inlineStr">
+        <is>
+          <t>AG House, Deira, Dubai</t>
+        </is>
+      </c>
+      <c r="I16" s="5" t="inlineStr">
+        <is>
+          <t>UAE</t>
+        </is>
+      </c>
+      <c r="J16" s="5" t="inlineStr">
+        <is>
+          <t>10,000+ across 4,300+ locations (company)</t>
+        </is>
+      </c>
+      <c r="K16" s="5" t="inlineStr">
+        <is>
+          <t>4,300+ service locations</t>
+        </is>
+      </c>
+      <c r="L16" s="5" t="inlineStr">
+        <is>
+          <t>Not published</t>
+        </is>
+      </c>
+      <c r="M16" s="5" t="inlineStr">
+        <is>
+          <t>approx. AED 750M to 1,100M</t>
+        </is>
+      </c>
+      <c r="N16" s="5" t="inlineStr">
+        <is>
+          <t>Not published</t>
+        </is>
+      </c>
+      <c r="O16" s="5" t="inlineStr">
+        <is>
+          <t>Retail, commercial and residential portfolios</t>
+        </is>
+      </c>
+      <c r="P16" s="5" t="inlineStr">
+        <is>
+          <t>One of the largest private Emirati IFM providers in Dubai</t>
+        </is>
+      </c>
+      <c r="Q16" s="5" t="inlineStr">
+        <is>
+          <t>No government or state shareholder found in public sources</t>
+        </is>
+      </c>
+      <c r="R16" s="5" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="S16" s="5" t="inlineStr">
+        <is>
+          <t>mefma.org (AG Facilities Solutions); zawya.com (Al Ghurair appoints AGFS CEO); zoominfo.com</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="5" t="n">
+        <v>16</v>
+      </c>
+      <c r="B17" s="6" t="inlineStr">
+        <is>
+          <t>OCS Middle East (OCS United Service Emirates LLC)</t>
+        </is>
+      </c>
+      <c r="C17" s="5" t="inlineStr">
+        <is>
+          <t>Integrated FM, MEP O&amp;M, commercial cleaning and housekeeping, security</t>
+        </is>
+      </c>
+      <c r="D17" s="5" t="inlineStr">
+        <is>
+          <t>OCS Group (UK), now owned by private equity firm CD&amp;R</t>
+        </is>
+      </c>
+      <c r="E17" s="5" t="inlineStr">
+        <is>
+          <t>British (parent)</t>
+        </is>
+      </c>
+      <c r="F17" s="5" t="inlineStr">
+        <is>
+          <t>Private (PE-owned)</t>
+        </is>
+      </c>
+      <c r="G17" s="5" t="inlineStr">
+        <is>
+          <t>Regional launch via JV with Tadmur Group</t>
+        </is>
+      </c>
+      <c r="H17" s="5" t="inlineStr">
+        <is>
+          <t>The Curve Building, Al Quoz, Dubai</t>
+        </is>
+      </c>
+      <c r="I17" s="5" t="inlineStr">
+        <is>
+          <t>UAE, Qatar</t>
+        </is>
+      </c>
+      <c r="J17" s="5" t="inlineStr">
+        <is>
+          <t>101 to 200 in UAE (aggregator); group 87,000+</t>
+        </is>
+      </c>
+      <c r="K17" s="5" t="inlineStr">
+        <is>
+          <t>Backed by a global FM group</t>
+        </is>
+      </c>
+      <c r="L17" s="5" t="inlineStr">
+        <is>
+          <t>Not published for UAE</t>
+        </is>
+      </c>
+      <c r="M17" s="5" t="inlineStr">
+        <is>
+          <t>approx. AED 8M to 22M</t>
+        </is>
+      </c>
+      <c r="N17" s="5" t="inlineStr">
+        <is>
+          <t>Not published</t>
+        </is>
+      </c>
+      <c r="O17" s="5" t="inlineStr">
+        <is>
+          <t>Corporate offices</t>
+        </is>
+      </c>
+      <c r="P17" s="5" t="inlineStr">
+        <is>
+          <t>International IFM with cleaning and security in Dubai</t>
+        </is>
+      </c>
+      <c r="Q17" s="5" t="inlineStr">
+        <is>
+          <t>No government or state shareholder found in public sources</t>
+        </is>
+      </c>
+      <c r="R17" s="5" t="inlineStr">
+        <is>
+          <t>Low to medium</t>
+        </is>
+      </c>
+      <c r="S17" s="5" t="inlineStr">
+        <is>
+          <t>bbgdubai.org (OCS Middle East); zawya.com (OCS enters Qatar); pulse2.com (OCS/Mitie)</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="5" t="n">
+        <v>17</v>
+      </c>
+      <c r="B18" s="6" t="inlineStr">
+        <is>
+          <t>BKA Facilities Management (formerly BK Gulf FM)</t>
+        </is>
+      </c>
+      <c r="C18" s="5" t="inlineStr">
+        <is>
+          <t>Integrated FM: MEP, building services, soft services</t>
+        </is>
+      </c>
+      <c r="D18" s="5" t="inlineStr">
+        <is>
+          <t>50/50 Dutco Group (Baker family) and Al Ali Property Investments</t>
+        </is>
+      </c>
+      <c r="E18" s="5" t="inlineStr">
+        <is>
+          <t>Emirati</t>
+        </is>
+      </c>
+      <c r="F18" s="5" t="inlineStr">
+        <is>
+          <t>Private</t>
+        </is>
+      </c>
+      <c r="G18" s="5" t="inlineStr">
+        <is>
+          <t>1998 (rebranded 2023)</t>
+        </is>
+      </c>
+      <c r="H18" s="5" t="inlineStr">
+        <is>
+          <t>Dubai</t>
+        </is>
+      </c>
+      <c r="I18" s="5" t="inlineStr">
+        <is>
+          <t>UAE</t>
+        </is>
+      </c>
+      <c r="J18" s="5" t="inlineStr">
+        <is>
+          <t>1,001 to 2,000 (aggregator); Dutco group 14,000+</t>
+        </is>
+      </c>
+      <c r="K18" s="5" t="inlineStr">
+        <is>
+          <t>Dutco bought out Balfour Beatty's 49% in 2017</t>
+        </is>
+      </c>
+      <c r="L18" s="5" t="inlineStr">
+        <is>
+          <t>Not published</t>
+        </is>
+      </c>
+      <c r="M18" s="5" t="inlineStr">
+        <is>
+          <t>approx. AED 75M to 220M</t>
+        </is>
+      </c>
+      <c r="N18" s="5" t="inlineStr">
+        <is>
+          <t>Not published</t>
+        </is>
+      </c>
+      <c r="O18" s="5" t="inlineStr">
+        <is>
+          <t>Commercial and residential buildings</t>
+        </is>
+      </c>
+      <c r="P18" s="5" t="inlineStr">
+        <is>
+          <t>Established Dubai IFM with MEP strength</t>
+        </is>
+      </c>
+      <c r="Q18" s="5" t="inlineStr">
+        <is>
+          <t>No government or state shareholder found in public sources</t>
+        </is>
+      </c>
+      <c r="R18" s="5" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="S18" s="5" t="inlineStr">
+        <is>
+          <t>dutco.com (BK Gulf FM); thenationalnews.com (Balfour Beatty sale); mefma.org (BKA FM)</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="5" t="n">
+        <v>18</v>
+      </c>
+      <c r="B19" s="6" t="inlineStr">
+        <is>
+          <t>Al Bonian Facilities Management</t>
+        </is>
+      </c>
+      <c r="C19" s="5" t="inlineStr">
+        <is>
+          <t>Hard FM, soft FM, security, engineering and specialist services</t>
+        </is>
+      </c>
+      <c r="D19" s="5" t="inlineStr">
+        <is>
+          <t>Private (Albonian International). Owner not published; CEO Ayman Salah Bustami</t>
+        </is>
+      </c>
+      <c r="E19" s="5" t="inlineStr">
+        <is>
+          <t>Not published</t>
+        </is>
+      </c>
+      <c r="F19" s="5" t="inlineStr">
+        <is>
+          <t>Private</t>
+        </is>
+      </c>
+      <c r="G19" s="5" t="inlineStr">
+        <is>
+          <t>2013</t>
+        </is>
+      </c>
+      <c r="H19" s="5" t="inlineStr">
+        <is>
+          <t>Dubai</t>
+        </is>
+      </c>
+      <c r="I19" s="5" t="inlineStr">
+        <is>
+          <t>UAE</t>
+        </is>
+      </c>
+      <c r="J19" s="5" t="inlineStr">
+        <is>
+          <t>125 to 500 (aggregator, conflicting)</t>
+        </is>
+      </c>
+      <c r="K19" s="5" t="inlineStr">
+        <is>
+          <t>Offers security in-house, like MEBS</t>
+        </is>
+      </c>
+      <c r="L19" s="5" t="inlineStr">
+        <is>
+          <t>Not published</t>
+        </is>
+      </c>
+      <c r="M19" s="5" t="inlineStr">
+        <is>
+          <t>approx. AED 9M to 55M</t>
+        </is>
+      </c>
+      <c r="N19" s="5" t="inlineStr">
+        <is>
+          <t>Not published</t>
+        </is>
+      </c>
+      <c r="O19" s="5" t="inlineStr">
+        <is>
+          <t>Commercial and residential</t>
+        </is>
+      </c>
+      <c r="P19" s="5" t="inlineStr">
+        <is>
+          <t>Dubai IFM bundling security and soft services</t>
+        </is>
+      </c>
+      <c r="Q19" s="5" t="inlineStr">
+        <is>
+          <t>No government or state shareholder found in public sources</t>
+        </is>
+      </c>
+      <c r="R19" s="5" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="S19" s="5" t="inlineStr">
+        <is>
+          <t>mefma.org (Al Bonian FM); cbnme.com; prospeo.io</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="5" t="n">
+        <v>19</v>
+      </c>
+      <c r="B20" s="6" t="inlineStr">
+        <is>
+          <t>iFM Facilities Management LLC</t>
+        </is>
+      </c>
+      <c r="C20" s="5" t="inlineStr">
+        <is>
+          <t>Smart integrated FM across all seven emirates</t>
+        </is>
+      </c>
+      <c r="D20" s="5" t="inlineStr">
+        <is>
+          <t>Private. CEO Hazem Al Hamed (aggregator). Owner not published</t>
+        </is>
+      </c>
+      <c r="E20" s="5" t="inlineStr">
+        <is>
+          <t>Not published</t>
+        </is>
+      </c>
+      <c r="F20" s="5" t="inlineStr">
+        <is>
+          <t>Private</t>
+        </is>
+      </c>
+      <c r="G20" s="5" t="inlineStr">
+        <is>
+          <t>Not published</t>
+        </is>
+      </c>
+      <c r="H20" s="5" t="inlineStr">
+        <is>
+          <t>Abu Dhabi / Dubai (sources conflict)</t>
+        </is>
+      </c>
+      <c r="I20" s="5" t="inlineStr">
+        <is>
+          <t>All seven emirates</t>
+        </is>
+      </c>
+      <c r="J20" s="5" t="inlineStr">
+        <is>
+          <t>201 to 600 (aggregators)</t>
+        </is>
+      </c>
+      <c r="K20" s="5" t="inlineStr">
+        <is>
+          <t>UAE-wide coverage</t>
+        </is>
+      </c>
+      <c r="L20" s="5" t="inlineStr">
+        <is>
+          <t>Not published</t>
+        </is>
+      </c>
+      <c r="M20" s="5" t="inlineStr">
+        <is>
+          <t>approx. AED 15M to 66M</t>
+        </is>
+      </c>
+      <c r="N20" s="5" t="inlineStr">
+        <is>
+          <t>Not published</t>
+        </is>
+      </c>
+      <c r="O20" s="5" t="inlineStr">
+        <is>
+          <t>Not published</t>
+        </is>
+      </c>
+      <c r="P20" s="5" t="inlineStr">
+        <is>
+          <t>UAE-wide IFM competitor</t>
+        </is>
+      </c>
+      <c r="Q20" s="5" t="inlineStr">
+        <is>
+          <t>No government or state shareholder found in public sources</t>
+        </is>
+      </c>
+      <c r="R20" s="5" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="S20" s="5" t="inlineStr">
+        <is>
+          <t>mefma.org (iFM); aeroleads.com; village.ai</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="5" t="n">
+        <v>20</v>
+      </c>
+      <c r="B21" s="6" t="inlineStr">
+        <is>
+          <t>QBG Services</t>
+        </is>
+      </c>
+      <c r="C21" s="5" t="inlineStr">
+        <is>
+          <t>Facilities management, staffing, landscaping</t>
+        </is>
+      </c>
+      <c r="D21" s="5" t="inlineStr">
+        <is>
+          <t>Qurum Business Group (Oman). Owners not published</t>
+        </is>
+      </c>
+      <c r="E21" s="5" t="inlineStr">
+        <is>
+          <t>Omani</t>
+        </is>
+      </c>
+      <c r="F21" s="5" t="inlineStr">
+        <is>
+          <t>Private group</t>
+        </is>
+      </c>
+      <c r="G21" s="5" t="inlineStr">
+        <is>
+          <t>Group 1970 (unverified)</t>
+        </is>
+      </c>
+      <c r="H21" s="5" t="inlineStr">
+        <is>
+          <t>Muscat, Oman (UAE operations in Dubai and Abu Dhabi)</t>
+        </is>
+      </c>
+      <c r="I21" s="5" t="inlineStr">
+        <is>
+          <t>UAE, Oman</t>
+        </is>
+      </c>
+      <c r="J21" s="5" t="inlineStr">
+        <is>
+          <t>51 to 280 (aggregators)</t>
+        </is>
+      </c>
+      <c r="K21" s="5" t="inlineStr">
+        <is>
+          <t>Staffing arm placed 150+ Emiratis on UAE projects</t>
+        </is>
+      </c>
+      <c r="L21" s="5" t="inlineStr">
+        <is>
+          <t>Not published</t>
+        </is>
+      </c>
+      <c r="M21" s="5" t="inlineStr">
+        <is>
+          <t>approx. AED 4M to 31M</t>
+        </is>
+      </c>
+      <c r="N21" s="5" t="inlineStr">
+        <is>
+          <t>Not published</t>
+        </is>
+      </c>
+      <c r="O21" s="5" t="inlineStr">
+        <is>
+          <t>Hospitality and commercial clients</t>
+        </is>
+      </c>
+      <c r="P21" s="5" t="inlineStr">
+        <is>
+          <t>FM and staffing competitor in Dubai and Abu Dhabi</t>
+        </is>
+      </c>
+      <c r="Q21" s="5" t="inlineStr">
+        <is>
+          <t>No government or state shareholder found in public sources</t>
+        </is>
+      </c>
+      <c r="R21" s="5" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="S21" s="5" t="inlineStr">
+        <is>
+          <t>village.do (QBG Services); protenders.com (Qurum Business Group); issuu.com</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:S9"/>
+  <autoFilter ref="A1:S21"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -1489,7 +2629,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:S7"/>
+  <dimension ref="A1:S21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="4" customWidth="1" min="1" max="1"/>
@@ -2180,8 +3320,1338 @@
         </is>
       </c>
     </row>
+    <row r="8">
+      <c r="A8" s="5" t="n">
+        <v>7</v>
+      </c>
+      <c r="B8" s="7" t="inlineStr">
+        <is>
+          <t>Emirates Security Services (Emirates Guard Services)</t>
+        </is>
+      </c>
+      <c r="C8" s="5" t="inlineStr">
+        <is>
+          <t>Manned guarding</t>
+        </is>
+      </c>
+      <c r="D8" s="5" t="inlineStr">
+        <is>
+          <t>Locally owned private company. Owner not published</t>
+        </is>
+      </c>
+      <c r="E8" s="5" t="inlineStr">
+        <is>
+          <t>Emirati</t>
+        </is>
+      </c>
+      <c r="F8" s="5" t="inlineStr">
+        <is>
+          <t>Private</t>
+        </is>
+      </c>
+      <c r="G8" s="5" t="inlineStr">
+        <is>
+          <t>2005</t>
+        </is>
+      </c>
+      <c r="H8" s="5" t="inlineStr">
+        <is>
+          <t>Abu Dhabi</t>
+        </is>
+      </c>
+      <c r="I8" s="5" t="inlineStr">
+        <is>
+          <t>UAE</t>
+        </is>
+      </c>
+      <c r="J8" s="5" t="inlineStr">
+        <is>
+          <t>5,001 to 10,000 (directory)</t>
+        </is>
+      </c>
+      <c r="K8" s="5" t="inlineStr">
+        <is>
+          <t>Calls itself the largest locally owned security company</t>
+        </is>
+      </c>
+      <c r="L8" s="5" t="inlineStr">
+        <is>
+          <t>Not published</t>
+        </is>
+      </c>
+      <c r="M8" s="5" t="inlineStr">
+        <is>
+          <t>approx. AED 360M to 1,000M</t>
+        </is>
+      </c>
+      <c r="N8" s="5" t="inlineStr">
+        <is>
+          <t>Abu Dhabi Police Security Support Services; federal licences</t>
+        </is>
+      </c>
+      <c r="O8" s="5" t="inlineStr">
+        <is>
+          <t>Not published</t>
+        </is>
+      </c>
+      <c r="P8" s="5" t="inlineStr">
+        <is>
+          <t>Large Abu Dhabi guarding competitor</t>
+        </is>
+      </c>
+      <c r="Q8" s="5" t="inlineStr">
+        <is>
+          <t>No government or state shareholder found in public sources</t>
+        </is>
+      </c>
+      <c r="R8" s="5" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="S8" s="5" t="inlineStr">
+        <is>
+          <t>naukrigulf.com (Emirates Security Services); kompass.com</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="5" t="n">
+        <v>8</v>
+      </c>
+      <c r="B9" s="7" t="inlineStr">
+        <is>
+          <t>United Security Group (USG)</t>
+        </is>
+      </c>
+      <c r="C9" s="5" t="inlineStr">
+        <is>
+          <t>Security guarding and mobile patrolling</t>
+        </is>
+      </c>
+      <c r="D9" s="5" t="inlineStr">
+        <is>
+          <t>Rashed Bin Khalaf Al Otaiba (per Naukri; another directory names different owners)</t>
+        </is>
+      </c>
+      <c r="E9" s="5" t="inlineStr">
+        <is>
+          <t>Emirati</t>
+        </is>
+      </c>
+      <c r="F9" s="5" t="inlineStr">
+        <is>
+          <t>Private</t>
+        </is>
+      </c>
+      <c r="G9" s="5" t="inlineStr">
+        <is>
+          <t>2007</t>
+        </is>
+      </c>
+      <c r="H9" s="5" t="inlineStr">
+        <is>
+          <t>Abu Dhabi (5 branches)</t>
+        </is>
+      </c>
+      <c r="I9" s="5" t="inlineStr">
+        <is>
+          <t>UAE</t>
+        </is>
+      </c>
+      <c r="J9" s="5" t="inlineStr">
+        <is>
+          <t>501 to 10,000 (sources conflict)</t>
+        </is>
+      </c>
+      <c r="K9" s="5" t="inlineStr">
+        <is>
+          <t>Five branch offices</t>
+        </is>
+      </c>
+      <c r="L9" s="5" t="inlineStr">
+        <is>
+          <t>US$10M to 50M (Naukri) vs US$172.6M (ZoomInfo), estimates</t>
+        </is>
+      </c>
+      <c r="M9" s="5" t="inlineStr">
+        <is>
+          <t>approx. AED 72M to 500M</t>
+        </is>
+      </c>
+      <c r="N9" s="5" t="inlineStr">
+        <is>
+          <t>Not published</t>
+        </is>
+      </c>
+      <c r="O9" s="5" t="inlineStr">
+        <is>
+          <t>Not published</t>
+        </is>
+      </c>
+      <c r="P9" s="5" t="inlineStr">
+        <is>
+          <t>One of the larger locally owned guarding firms</t>
+        </is>
+      </c>
+      <c r="Q9" s="5" t="inlineStr">
+        <is>
+          <t>No government or state shareholder found in public sources</t>
+        </is>
+      </c>
+      <c r="R9" s="5" t="inlineStr">
+        <is>
+          <t>Low to medium</t>
+        </is>
+      </c>
+      <c r="S9" s="5" t="inlineStr">
+        <is>
+          <t>naukrigulf.com (United Security Group); zoominfo.com; indeed.com</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="5" t="n">
+        <v>9</v>
+      </c>
+      <c r="B10" s="7" t="inlineStr">
+        <is>
+          <t>Emirates Gateway Security Services (EGSS)</t>
+        </is>
+      </c>
+      <c r="C10" s="5" t="inlineStr">
+        <is>
+          <t>Manned guarding</t>
+        </is>
+      </c>
+      <c r="D10" s="5" t="inlineStr">
+        <is>
+          <t>Private. Owner not published</t>
+        </is>
+      </c>
+      <c r="E10" s="5" t="inlineStr">
+        <is>
+          <t>Not published</t>
+        </is>
+      </c>
+      <c r="F10" s="5" t="inlineStr">
+        <is>
+          <t>Private</t>
+        </is>
+      </c>
+      <c r="G10" s="5" t="inlineStr">
+        <is>
+          <t>2007</t>
+        </is>
+      </c>
+      <c r="H10" s="5" t="inlineStr">
+        <is>
+          <t>Abu Dhabi</t>
+        </is>
+      </c>
+      <c r="I10" s="5" t="inlineStr">
+        <is>
+          <t>UAE</t>
+        </is>
+      </c>
+      <c r="J10" s="5" t="inlineStr">
+        <is>
+          <t>166 to 500 (aggregator)</t>
+        </is>
+      </c>
+      <c r="K10" s="5" t="inlineStr">
+        <is>
+          <t>Abu Dhabi guarding</t>
+        </is>
+      </c>
+      <c r="L10" s="5" t="inlineStr">
+        <is>
+          <t>Not published</t>
+        </is>
+      </c>
+      <c r="M10" s="5" t="inlineStr">
+        <is>
+          <t>approx. AED 12M to 50M</t>
+        </is>
+      </c>
+      <c r="N10" s="5" t="inlineStr">
+        <is>
+          <t>Not published</t>
+        </is>
+      </c>
+      <c r="O10" s="5" t="inlineStr">
+        <is>
+          <t>Not published</t>
+        </is>
+      </c>
+      <c r="P10" s="5" t="inlineStr">
+        <is>
+          <t>Abu Dhabi guarding competitor</t>
+        </is>
+      </c>
+      <c r="Q10" s="5" t="inlineStr">
+        <is>
+          <t>No government or state shareholder found in public sources</t>
+        </is>
+      </c>
+      <c r="R10" s="5" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="S10" s="5" t="inlineStr">
+        <is>
+          <t>prospeo.io (EGSS); propertyfinder.ae</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="5" t="n">
+        <v>10</v>
+      </c>
+      <c r="B11" s="7" t="inlineStr">
+        <is>
+          <t>Al Falah Security Services</t>
+        </is>
+      </c>
+      <c r="C11" s="5" t="inlineStr">
+        <is>
+          <t>Guarding, access control, perimeter patrols, electronic security operations, 24/7 operations centre</t>
+        </is>
+      </c>
+      <c r="D11" s="5" t="inlineStr">
+        <is>
+          <t>Private. Owner not published</t>
+        </is>
+      </c>
+      <c r="E11" s="5" t="inlineStr">
+        <is>
+          <t>Not published</t>
+        </is>
+      </c>
+      <c r="F11" s="5" t="inlineStr">
+        <is>
+          <t>Private</t>
+        </is>
+      </c>
+      <c r="G11" s="5" t="inlineStr">
+        <is>
+          <t>Not published</t>
+        </is>
+      </c>
+      <c r="H11" s="5" t="inlineStr">
+        <is>
+          <t>Mussafah, Abu Dhabi</t>
+        </is>
+      </c>
+      <c r="I11" s="5" t="inlineStr">
+        <is>
+          <t>UAE</t>
+        </is>
+      </c>
+      <c r="J11" s="5" t="inlineStr">
+        <is>
+          <t>Not published</t>
+        </is>
+      </c>
+      <c r="K11" s="5" t="inlineStr">
+        <is>
+          <t>24/7 operations centre</t>
+        </is>
+      </c>
+      <c r="L11" s="5" t="inlineStr">
+        <is>
+          <t>Not published</t>
+        </is>
+      </c>
+      <c r="M11" s="5" t="inlineStr">
+        <is>
+          <t>Cannot estimate (headcount unknown)</t>
+        </is>
+      </c>
+      <c r="N11" s="5" t="inlineStr">
+        <is>
+          <t>Not published</t>
+        </is>
+      </c>
+      <c r="O11" s="5" t="inlineStr">
+        <is>
+          <t>Not published</t>
+        </is>
+      </c>
+      <c r="P11" s="5" t="inlineStr">
+        <is>
+          <t>Abu Dhabi guarding competitor</t>
+        </is>
+      </c>
+      <c r="Q11" s="5" t="inlineStr">
+        <is>
+          <t>No government or state shareholder found in public sources</t>
+        </is>
+      </c>
+      <c r="R11" s="5" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="S11" s="5" t="inlineStr">
+        <is>
+          <t>naukrigulf.com (Al Falah Security Services)</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="5" t="n">
+        <v>11</v>
+      </c>
+      <c r="B12" s="7" t="inlineStr">
+        <is>
+          <t>RANN Security Services</t>
+        </is>
+      </c>
+      <c r="C12" s="5" t="inlineStr">
+        <is>
+          <t>Guarding, remote monitoring, risk assessments, virtual guarding, field supervision</t>
+        </is>
+      </c>
+      <c r="D12" s="5" t="inlineStr">
+        <is>
+          <t>Private. Owner not published</t>
+        </is>
+      </c>
+      <c r="E12" s="5" t="inlineStr">
+        <is>
+          <t>Not published</t>
+        </is>
+      </c>
+      <c r="F12" s="5" t="inlineStr">
+        <is>
+          <t>Private</t>
+        </is>
+      </c>
+      <c r="G12" s="5" t="inlineStr">
+        <is>
+          <t>Not published</t>
+        </is>
+      </c>
+      <c r="H12" s="5" t="inlineStr">
+        <is>
+          <t>Al Rigga, Dubai</t>
+        </is>
+      </c>
+      <c r="I12" s="5" t="inlineStr">
+        <is>
+          <t>UAE</t>
+        </is>
+      </c>
+      <c r="J12" s="5" t="inlineStr">
+        <is>
+          <t>Not published</t>
+        </is>
+      </c>
+      <c r="K12" s="5" t="inlineStr">
+        <is>
+          <t>Claims to be a large SIRA-certified firm</t>
+        </is>
+      </c>
+      <c r="L12" s="5" t="inlineStr">
+        <is>
+          <t>Not published</t>
+        </is>
+      </c>
+      <c r="M12" s="5" t="inlineStr">
+        <is>
+          <t>Cannot estimate (headcount unknown)</t>
+        </is>
+      </c>
+      <c r="N12" s="5" t="inlineStr">
+        <is>
+          <t>ISO 9001:2008 (per listing)</t>
+        </is>
+      </c>
+      <c r="O12" s="5" t="inlineStr">
+        <is>
+          <t>Not published</t>
+        </is>
+      </c>
+      <c r="P12" s="5" t="inlineStr">
+        <is>
+          <t>Dubai guarding competitor</t>
+        </is>
+      </c>
+      <c r="Q12" s="5" t="inlineStr">
+        <is>
+          <t>No government or state shareholder found in public sources</t>
+        </is>
+      </c>
+      <c r="R12" s="5" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="S12" s="5" t="inlineStr">
+        <is>
+          <t>bayut.com (security companies); hidubai.com</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="5" t="n">
+        <v>12</v>
+      </c>
+      <c r="B13" s="7" t="inlineStr">
+        <is>
+          <t>Black Horse Security Services</t>
+        </is>
+      </c>
+      <c r="C13" s="5" t="inlineStr">
+        <is>
+          <t>Guarding and patrol for events, retail and residential</t>
+        </is>
+      </c>
+      <c r="D13" s="5" t="inlineStr">
+        <is>
+          <t>Wael Ahmed (per Prospeo, unverified)</t>
+        </is>
+      </c>
+      <c r="E13" s="5" t="inlineStr">
+        <is>
+          <t>Not published</t>
+        </is>
+      </c>
+      <c r="F13" s="5" t="inlineStr">
+        <is>
+          <t>Private</t>
+        </is>
+      </c>
+      <c r="G13" s="5" t="inlineStr">
+        <is>
+          <t>2007</t>
+        </is>
+      </c>
+      <c r="H13" s="5" t="inlineStr">
+        <is>
+          <t>Port Saeed, Dubai</t>
+        </is>
+      </c>
+      <c r="I13" s="5" t="inlineStr">
+        <is>
+          <t>UAE</t>
+        </is>
+      </c>
+      <c r="J13" s="5" t="inlineStr">
+        <is>
+          <t>21 to 50 (aggregator)</t>
+        </is>
+      </c>
+      <c r="K13" s="5" t="inlineStr">
+        <is>
+          <t>Events, hospitals, hotels</t>
+        </is>
+      </c>
+      <c r="L13" s="5" t="inlineStr">
+        <is>
+          <t>Not published</t>
+        </is>
+      </c>
+      <c r="M13" s="5" t="inlineStr">
+        <is>
+          <t>approx. AED 2M to 5M</t>
+        </is>
+      </c>
+      <c r="N13" s="5" t="inlineStr">
+        <is>
+          <t>Not published</t>
+        </is>
+      </c>
+      <c r="O13" s="5" t="inlineStr">
+        <is>
+          <t>Events, hospitals, hotels</t>
+        </is>
+      </c>
+      <c r="P13" s="5" t="inlineStr">
+        <is>
+          <t>Small Dubai guarding competitor</t>
+        </is>
+      </c>
+      <c r="Q13" s="5" t="inlineStr">
+        <is>
+          <t>No government or state shareholder found in public sources</t>
+        </is>
+      </c>
+      <c r="R13" s="5" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="S13" s="5" t="inlineStr">
+        <is>
+          <t>sothebysrealty.ae (security companies); hidubai.com; prospeo.io</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="5" t="n">
+        <v>13</v>
+      </c>
+      <c r="B14" s="7" t="inlineStr">
+        <is>
+          <t>Doorsec Security Services LLC</t>
+        </is>
+      </c>
+      <c r="C14" s="5" t="inlineStr">
+        <is>
+          <t>Manned guarding</t>
+        </is>
+      </c>
+      <c r="D14" s="5" t="inlineStr">
+        <is>
+          <t>Private. Owner not published</t>
+        </is>
+      </c>
+      <c r="E14" s="5" t="inlineStr">
+        <is>
+          <t>Not published</t>
+        </is>
+      </c>
+      <c r="F14" s="5" t="inlineStr">
+        <is>
+          <t>Private</t>
+        </is>
+      </c>
+      <c r="G14" s="5" t="inlineStr">
+        <is>
+          <t>2012</t>
+        </is>
+      </c>
+      <c r="H14" s="5" t="inlineStr">
+        <is>
+          <t>Dubai</t>
+        </is>
+      </c>
+      <c r="I14" s="5" t="inlineStr">
+        <is>
+          <t>UAE</t>
+        </is>
+      </c>
+      <c r="J14" s="5" t="inlineStr">
+        <is>
+          <t>42 to 100 (aggregator)</t>
+        </is>
+      </c>
+      <c r="K14" s="5" t="inlineStr">
+        <is>
+          <t>Hires directly</t>
+        </is>
+      </c>
+      <c r="L14" s="5" t="inlineStr">
+        <is>
+          <t>Not published</t>
+        </is>
+      </c>
+      <c r="M14" s="5" t="inlineStr">
+        <is>
+          <t>approx. AED 3M to 10M</t>
+        </is>
+      </c>
+      <c r="N14" s="5" t="inlineStr">
+        <is>
+          <t>Not confirmed</t>
+        </is>
+      </c>
+      <c r="O14" s="5" t="inlineStr">
+        <is>
+          <t>Not published</t>
+        </is>
+      </c>
+      <c r="P14" s="5" t="inlineStr">
+        <is>
+          <t>Dubai guarding competitor</t>
+        </is>
+      </c>
+      <c r="Q14" s="5" t="inlineStr">
+        <is>
+          <t>No government or state shareholder found in public sources</t>
+        </is>
+      </c>
+      <c r="R14" s="5" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="S14" s="5" t="inlineStr">
+        <is>
+          <t>prospeo.io (Doorsec); ae.indeed.com</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="5" t="n">
+        <v>14</v>
+      </c>
+      <c r="B15" s="7" t="inlineStr">
+        <is>
+          <t>Westminster Security UAE</t>
+        </is>
+      </c>
+      <c r="C15" s="5" t="inlineStr">
+        <is>
+          <t>Close protection, security advance teams, chauffeurs, counter-surveillance, residential security</t>
+        </is>
+      </c>
+      <c r="D15" s="5" t="inlineStr">
+        <is>
+          <t>Westminster Security Group (UK, private; CEO John Moore)</t>
+        </is>
+      </c>
+      <c r="E15" s="5" t="inlineStr">
+        <is>
+          <t>British (parent)</t>
+        </is>
+      </c>
+      <c r="F15" s="5" t="inlineStr">
+        <is>
+          <t>Private</t>
+        </is>
+      </c>
+      <c r="G15" s="5" t="inlineStr">
+        <is>
+          <t>2024</t>
+        </is>
+      </c>
+      <c r="H15" s="5" t="inlineStr">
+        <is>
+          <t>Dubai</t>
+        </is>
+      </c>
+      <c r="I15" s="5" t="inlineStr">
+        <is>
+          <t>UAE</t>
+        </is>
+      </c>
+      <c r="J15" s="5" t="inlineStr">
+        <is>
+          <t>Not published</t>
+        </is>
+      </c>
+      <c r="K15" s="5" t="inlineStr">
+        <is>
+          <t>High-net-worth and family office clients</t>
+        </is>
+      </c>
+      <c r="L15" s="5" t="inlineStr">
+        <is>
+          <t>Not published</t>
+        </is>
+      </c>
+      <c r="M15" s="5" t="inlineStr">
+        <is>
+          <t>Cannot estimate (headcount unknown)</t>
+        </is>
+      </c>
+      <c r="N15" s="5" t="inlineStr">
+        <is>
+          <t>Not published</t>
+        </is>
+      </c>
+      <c r="O15" s="5" t="inlineStr">
+        <is>
+          <t>Private families and individuals</t>
+        </is>
+      </c>
+      <c r="P15" s="5" t="inlineStr">
+        <is>
+          <t>Premium security competitor for VIP and residential work</t>
+        </is>
+      </c>
+      <c r="Q15" s="5" t="inlineStr">
+        <is>
+          <t>No government or state shareholder found in public sources</t>
+        </is>
+      </c>
+      <c r="R15" s="5" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="S15" s="5" t="inlineStr">
+        <is>
+          <t>westminstersecurity.co.uk (Dubai launch); securitysystemsnews.com</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="5" t="n">
+        <v>15</v>
+      </c>
+      <c r="B16" s="7" t="inlineStr">
+        <is>
+          <t>Belhasa Falcon (formerly BELCOM)</t>
+        </is>
+      </c>
+      <c r="C16" s="5" t="inlineStr">
+        <is>
+          <t>Private security guarding</t>
+        </is>
+      </c>
+      <c r="D16" s="5" t="inlineStr">
+        <is>
+          <t>Belhasa Group of Companies</t>
+        </is>
+      </c>
+      <c r="E16" s="5" t="inlineStr">
+        <is>
+          <t>Emirati</t>
+        </is>
+      </c>
+      <c r="F16" s="5" t="inlineStr">
+        <is>
+          <t>Private family group</t>
+        </is>
+      </c>
+      <c r="G16" s="5" t="inlineStr">
+        <is>
+          <t>1993 or 1995 (sources conflict)</t>
+        </is>
+      </c>
+      <c r="H16" s="5" t="inlineStr">
+        <is>
+          <t>Dubai</t>
+        </is>
+      </c>
+      <c r="I16" s="5" t="inlineStr">
+        <is>
+          <t>UAE</t>
+        </is>
+      </c>
+      <c r="J16" s="5" t="inlineStr">
+        <is>
+          <t>Not published</t>
+        </is>
+      </c>
+      <c r="K16" s="5" t="inlineStr">
+        <is>
+          <t>Part of Belhasa Group</t>
+        </is>
+      </c>
+      <c r="L16" s="5" t="inlineStr">
+        <is>
+          <t>Not published</t>
+        </is>
+      </c>
+      <c r="M16" s="5" t="inlineStr">
+        <is>
+          <t>Cannot estimate (headcount unknown)</t>
+        </is>
+      </c>
+      <c r="N16" s="5" t="inlineStr">
+        <is>
+          <t>Not published</t>
+        </is>
+      </c>
+      <c r="O16" s="5" t="inlineStr">
+        <is>
+          <t>Not published</t>
+        </is>
+      </c>
+      <c r="P16" s="5" t="inlineStr">
+        <is>
+          <t>Emirati family-owned Dubai guarding firm</t>
+        </is>
+      </c>
+      <c r="Q16" s="5" t="inlineStr">
+        <is>
+          <t>No government or state shareholder found in public sources</t>
+        </is>
+      </c>
+      <c r="R16" s="5" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="S16" s="5" t="inlineStr">
+        <is>
+          <t>naukrigulf.com (Belhasa Falcon)</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="5" t="n">
+        <v>16</v>
+      </c>
+      <c r="B17" s="7" t="inlineStr">
+        <is>
+          <t>Fursan Security Services LLC</t>
+        </is>
+      </c>
+      <c r="C17" s="5" t="inlineStr">
+        <is>
+          <t>Manned guarding and mobile security</t>
+        </is>
+      </c>
+      <c r="D17" s="5" t="inlineStr">
+        <is>
+          <t>Private. Owner not published</t>
+        </is>
+      </c>
+      <c r="E17" s="5" t="inlineStr">
+        <is>
+          <t>Not published</t>
+        </is>
+      </c>
+      <c r="F17" s="5" t="inlineStr">
+        <is>
+          <t>Private</t>
+        </is>
+      </c>
+      <c r="G17" s="5" t="inlineStr">
+        <is>
+          <t>2014</t>
+        </is>
+      </c>
+      <c r="H17" s="5" t="inlineStr">
+        <is>
+          <t>Abu Dhabi</t>
+        </is>
+      </c>
+      <c r="I17" s="5" t="inlineStr">
+        <is>
+          <t>UAE</t>
+        </is>
+      </c>
+      <c r="J17" s="5" t="inlineStr">
+        <is>
+          <t>20 to 29 (aggregators)</t>
+        </is>
+      </c>
+      <c r="K17" s="5" t="inlineStr">
+        <is>
+          <t>Small guarding firm</t>
+        </is>
+      </c>
+      <c r="L17" s="5" t="inlineStr">
+        <is>
+          <t>Not published</t>
+        </is>
+      </c>
+      <c r="M17" s="5" t="inlineStr">
+        <is>
+          <t>approx. AED 1M to 3M</t>
+        </is>
+      </c>
+      <c r="N17" s="5" t="inlineStr">
+        <is>
+          <t>Not published</t>
+        </is>
+      </c>
+      <c r="O17" s="5" t="inlineStr">
+        <is>
+          <t>Not published</t>
+        </is>
+      </c>
+      <c r="P17" s="5" t="inlineStr">
+        <is>
+          <t>Small Abu Dhabi guarding competitor</t>
+        </is>
+      </c>
+      <c r="Q17" s="5" t="inlineStr">
+        <is>
+          <t>No government or state shareholder found in public sources</t>
+        </is>
+      </c>
+      <c r="R17" s="5" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="S17" s="5" t="inlineStr">
+        <is>
+          <t>village.ai (Fursan Security Services); aeroleads.com</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="5" t="n">
+        <v>17</v>
+      </c>
+      <c r="B18" s="7" t="inlineStr">
+        <is>
+          <t>Focus Security Services UAE</t>
+        </is>
+      </c>
+      <c r="C18" s="5" t="inlineStr">
+        <is>
+          <t>Manned guarding</t>
+        </is>
+      </c>
+      <c r="D18" s="5" t="inlineStr">
+        <is>
+          <t>Private. Owner not published</t>
+        </is>
+      </c>
+      <c r="E18" s="5" t="inlineStr">
+        <is>
+          <t>Not published</t>
+        </is>
+      </c>
+      <c r="F18" s="5" t="inlineStr">
+        <is>
+          <t>Private</t>
+        </is>
+      </c>
+      <c r="G18" s="5" t="inlineStr">
+        <is>
+          <t>2017</t>
+        </is>
+      </c>
+      <c r="H18" s="5" t="inlineStr">
+        <is>
+          <t>Ajman</t>
+        </is>
+      </c>
+      <c r="I18" s="5" t="inlineStr">
+        <is>
+          <t>UAE</t>
+        </is>
+      </c>
+      <c r="J18" s="5" t="inlineStr">
+        <is>
+          <t>58 to 200 (aggregator)</t>
+        </is>
+      </c>
+      <c r="K18" s="5" t="inlineStr">
+        <is>
+          <t>Northern emirates guarding</t>
+        </is>
+      </c>
+      <c r="L18" s="5" t="inlineStr">
+        <is>
+          <t>Not published</t>
+        </is>
+      </c>
+      <c r="M18" s="5" t="inlineStr">
+        <is>
+          <t>approx. AED 4M to 20M</t>
+        </is>
+      </c>
+      <c r="N18" s="5" t="inlineStr">
+        <is>
+          <t>Not published</t>
+        </is>
+      </c>
+      <c r="O18" s="5" t="inlineStr">
+        <is>
+          <t>Not published</t>
+        </is>
+      </c>
+      <c r="P18" s="5" t="inlineStr">
+        <is>
+          <t>Guarding competitor in the northern emirates</t>
+        </is>
+      </c>
+      <c r="Q18" s="5" t="inlineStr">
+        <is>
+          <t>No government or state shareholder found in public sources</t>
+        </is>
+      </c>
+      <c r="R18" s="5" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="S18" s="5" t="inlineStr">
+        <is>
+          <t>prospeo.io (Focus Security Services UAE)</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="5" t="n">
+        <v>18</v>
+      </c>
+      <c r="B19" s="7" t="inlineStr">
+        <is>
+          <t>Hawk Security Services LLC</t>
+        </is>
+      </c>
+      <c r="C19" s="5" t="inlineStr">
+        <is>
+          <t>Physical guarding, housekeeping, kitchen duct cleaning, office support</t>
+        </is>
+      </c>
+      <c r="D19" s="5" t="inlineStr">
+        <is>
+          <t>Private. Owner not published</t>
+        </is>
+      </c>
+      <c r="E19" s="5" t="inlineStr">
+        <is>
+          <t>Not published</t>
+        </is>
+      </c>
+      <c r="F19" s="5" t="inlineStr">
+        <is>
+          <t>Private</t>
+        </is>
+      </c>
+      <c r="G19" s="5" t="inlineStr">
+        <is>
+          <t>Not published</t>
+        </is>
+      </c>
+      <c r="H19" s="5" t="inlineStr">
+        <is>
+          <t>Garhoud, Dubai</t>
+        </is>
+      </c>
+      <c r="I19" s="5" t="inlineStr">
+        <is>
+          <t>All emirates</t>
+        </is>
+      </c>
+      <c r="J19" s="5" t="inlineStr">
+        <is>
+          <t>1,200+ (company); 11 to 50 (ZoomInfo)</t>
+        </is>
+      </c>
+      <c r="K19" s="5" t="inlineStr">
+        <is>
+          <t>Security plus housekeeping, close to MEBS's mix</t>
+        </is>
+      </c>
+      <c r="L19" s="5" t="inlineStr">
+        <is>
+          <t>Not published</t>
+        </is>
+      </c>
+      <c r="M19" s="5" t="inlineStr">
+        <is>
+          <t>approx. AED 72M to 120M</t>
+        </is>
+      </c>
+      <c r="N19" s="5" t="inlineStr">
+        <is>
+          <t>Not published</t>
+        </is>
+      </c>
+      <c r="O19" s="5" t="inlineStr">
+        <is>
+          <t>Not published</t>
+        </is>
+      </c>
+      <c r="P19" s="5" t="inlineStr">
+        <is>
+          <t>Bundles security and housekeeping like MEBS</t>
+        </is>
+      </c>
+      <c r="Q19" s="5" t="inlineStr">
+        <is>
+          <t>No government or state shareholder found in public sources</t>
+        </is>
+      </c>
+      <c r="R19" s="5" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="S19" s="5" t="inlineStr">
+        <is>
+          <t>naukrigulf.com (Hawk Security Services); kompass.com</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="5" t="n">
+        <v>19</v>
+      </c>
+      <c r="B20" s="7" t="inlineStr">
+        <is>
+          <t>Severity Security &amp; Guarding Services LLC</t>
+        </is>
+      </c>
+      <c r="C20" s="5" t="inlineStr">
+        <is>
+          <t>Manned guarding, hospitality security</t>
+        </is>
+      </c>
+      <c r="D20" s="5" t="inlineStr">
+        <is>
+          <t>Private. Owner not published</t>
+        </is>
+      </c>
+      <c r="E20" s="5" t="inlineStr">
+        <is>
+          <t>Not published</t>
+        </is>
+      </c>
+      <c r="F20" s="5" t="inlineStr">
+        <is>
+          <t>Private</t>
+        </is>
+      </c>
+      <c r="G20" s="5" t="inlineStr">
+        <is>
+          <t>Not published</t>
+        </is>
+      </c>
+      <c r="H20" s="5" t="inlineStr">
+        <is>
+          <t>Dubai</t>
+        </is>
+      </c>
+      <c r="I20" s="5" t="inlineStr">
+        <is>
+          <t>UAE</t>
+        </is>
+      </c>
+      <c r="J20" s="5" t="inlineStr">
+        <is>
+          <t>Not published</t>
+        </is>
+      </c>
+      <c r="K20" s="5" t="inlineStr">
+        <is>
+          <t>Hospitality-focused</t>
+        </is>
+      </c>
+      <c r="L20" s="5" t="inlineStr">
+        <is>
+          <t>Not published</t>
+        </is>
+      </c>
+      <c r="M20" s="5" t="inlineStr">
+        <is>
+          <t>Cannot estimate (headcount unknown)</t>
+        </is>
+      </c>
+      <c r="N20" s="5" t="inlineStr">
+        <is>
+          <t>SIRA (per listings)</t>
+        </is>
+      </c>
+      <c r="O20" s="5" t="inlineStr">
+        <is>
+          <t>Hospitality</t>
+        </is>
+      </c>
+      <c r="P20" s="5" t="inlineStr">
+        <is>
+          <t>Dubai guarding competitor in hospitality</t>
+        </is>
+      </c>
+      <c r="Q20" s="5" t="inlineStr">
+        <is>
+          <t>No government or state shareholder found in public sources</t>
+        </is>
+      </c>
+      <c r="R20" s="5" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="S20" s="5" t="inlineStr">
+        <is>
+          <t>severitysecurity.ae; thetalentpoint.com</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="5" t="n">
+        <v>20</v>
+      </c>
+      <c r="B21" s="7" t="inlineStr">
+        <is>
+          <t>Blue Diamond Facilities Management Services LLC</t>
+        </is>
+      </c>
+      <c r="C21" s="5" t="inlineStr">
+        <is>
+          <t>SIRA-approved guarding (part of Blue Diamond group, which also offers FM and cleaning)</t>
+        </is>
+      </c>
+      <c r="D21" s="5" t="inlineStr">
+        <is>
+          <t>Private (Blue Diamond Group). Owner not published</t>
+        </is>
+      </c>
+      <c r="E21" s="5" t="inlineStr">
+        <is>
+          <t>Not published</t>
+        </is>
+      </c>
+      <c r="F21" s="5" t="inlineStr">
+        <is>
+          <t>Private</t>
+        </is>
+      </c>
+      <c r="G21" s="5" t="inlineStr">
+        <is>
+          <t>2012 (group 1995)</t>
+        </is>
+      </c>
+      <c r="H21" s="5" t="inlineStr">
+        <is>
+          <t>Business Bay, Dubai</t>
+        </is>
+      </c>
+      <c r="I21" s="5" t="inlineStr">
+        <is>
+          <t>UAE</t>
+        </is>
+      </c>
+      <c r="J21" s="5" t="inlineStr">
+        <is>
+          <t>27 to 100 (aggregator)</t>
+        </is>
+      </c>
+      <c r="K21" s="5" t="inlineStr">
+        <is>
+          <t>Guards trained at Dubai Police-approved institutes</t>
+        </is>
+      </c>
+      <c r="L21" s="5" t="inlineStr">
+        <is>
+          <t>Not published</t>
+        </is>
+      </c>
+      <c r="M21" s="5" t="inlineStr">
+        <is>
+          <t>approx. AED 2M to 10M</t>
+        </is>
+      </c>
+      <c r="N21" s="5" t="inlineStr">
+        <is>
+          <t>SIRA; ISO 9001, 14001, 45001</t>
+        </is>
+      </c>
+      <c r="O21" s="5" t="inlineStr">
+        <is>
+          <t>Not published</t>
+        </is>
+      </c>
+      <c r="P21" s="5" t="inlineStr">
+        <is>
+          <t>Dubai security firm in a group that also does FM and cleaning</t>
+        </is>
+      </c>
+      <c r="Q21" s="5" t="inlineStr">
+        <is>
+          <t>No government or state shareholder found in public sources</t>
+        </is>
+      </c>
+      <c r="R21" s="5" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="S21" s="5" t="inlineStr">
+        <is>
+          <t>dubizzle.com (security companies); prospeo.io; village.ai</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:S7"/>
+  <autoFilter ref="A1:S21"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -2192,7 +4662,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:S7"/>
+  <dimension ref="A1:S21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="4" customWidth="1" min="1" max="1"/>
@@ -2883,8 +5353,1338 @@
         </is>
       </c>
     </row>
+    <row r="8">
+      <c r="A8" s="5" t="n">
+        <v>7</v>
+      </c>
+      <c r="B8" s="8" t="inlineStr">
+        <is>
+          <t>Cleanpro Facilities Management Services LLC</t>
+        </is>
+      </c>
+      <c r="C8" s="5" t="inlineStr">
+        <is>
+          <t>Cleaning and facility services</t>
+        </is>
+      </c>
+      <c r="D8" s="5" t="inlineStr">
+        <is>
+          <t>Private. Owner not published</t>
+        </is>
+      </c>
+      <c r="E8" s="5" t="inlineStr">
+        <is>
+          <t>Not published</t>
+        </is>
+      </c>
+      <c r="F8" s="5" t="inlineStr">
+        <is>
+          <t>Private</t>
+        </is>
+      </c>
+      <c r="G8" s="5" t="inlineStr">
+        <is>
+          <t>2013</t>
+        </is>
+      </c>
+      <c r="H8" s="5" t="inlineStr">
+        <is>
+          <t>Abu Dhabi (branch in Garhoud, Dubai)</t>
+        </is>
+      </c>
+      <c r="I8" s="5" t="inlineStr">
+        <is>
+          <t>UAE</t>
+        </is>
+      </c>
+      <c r="J8" s="5" t="inlineStr">
+        <is>
+          <t>Not published</t>
+        </is>
+      </c>
+      <c r="K8" s="5" t="inlineStr">
+        <is>
+          <t>Branches in Abu Dhabi and Dubai</t>
+        </is>
+      </c>
+      <c r="L8" s="5" t="inlineStr">
+        <is>
+          <t>Not published</t>
+        </is>
+      </c>
+      <c r="M8" s="5" t="inlineStr">
+        <is>
+          <t>Cannot estimate (headcount unknown)</t>
+        </is>
+      </c>
+      <c r="N8" s="5" t="inlineStr">
+        <is>
+          <t>Not published</t>
+        </is>
+      </c>
+      <c r="O8" s="5" t="inlineStr">
+        <is>
+          <t>Not published</t>
+        </is>
+      </c>
+      <c r="P8" s="5" t="inlineStr">
+        <is>
+          <t>Cleaning-led competitor in Abu Dhabi and Dubai</t>
+        </is>
+      </c>
+      <c r="Q8" s="5" t="inlineStr">
+        <is>
+          <t>No government or state shareholder found in public sources</t>
+        </is>
+      </c>
+      <c r="R8" s="5" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="S8" s="5" t="inlineStr">
+        <is>
+          <t>mefma.org (Cleanpro FMS); yellowpages-uae.com</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="5" t="n">
+        <v>8</v>
+      </c>
+      <c r="B9" s="8" t="inlineStr">
+        <is>
+          <t>WECARE Building Cleaning</t>
+        </is>
+      </c>
+      <c r="C9" s="5" t="inlineStr">
+        <is>
+          <t>Building cleaning</t>
+        </is>
+      </c>
+      <c r="D9" s="5" t="inlineStr">
+        <is>
+          <t>WECARE business group. Owner not published</t>
+        </is>
+      </c>
+      <c r="E9" s="5" t="inlineStr">
+        <is>
+          <t>Not published</t>
+        </is>
+      </c>
+      <c r="F9" s="5" t="inlineStr">
+        <is>
+          <t>Private</t>
+        </is>
+      </c>
+      <c r="G9" s="5" t="inlineStr">
+        <is>
+          <t>1997</t>
+        </is>
+      </c>
+      <c r="H9" s="5" t="inlineStr">
+        <is>
+          <t>Dubai</t>
+        </is>
+      </c>
+      <c r="I9" s="5" t="inlineStr">
+        <is>
+          <t>UAE</t>
+        </is>
+      </c>
+      <c r="J9" s="5" t="inlineStr">
+        <is>
+          <t>1,000+ (Dubai Govt HR listing)</t>
+        </is>
+      </c>
+      <c r="K9" s="5" t="inlineStr">
+        <is>
+          <t>Nationwide workforce</t>
+        </is>
+      </c>
+      <c r="L9" s="5" t="inlineStr">
+        <is>
+          <t>Not published</t>
+        </is>
+      </c>
+      <c r="M9" s="5" t="inlineStr">
+        <is>
+          <t>approx. AED 45M to 65M</t>
+        </is>
+      </c>
+      <c r="N9" s="5" t="inlineStr">
+        <is>
+          <t>Not published</t>
+        </is>
+      </c>
+      <c r="O9" s="5" t="inlineStr">
+        <is>
+          <t>Not published</t>
+        </is>
+      </c>
+      <c r="P9" s="5" t="inlineStr">
+        <is>
+          <t>Established Dubai building-cleaning contractor</t>
+        </is>
+      </c>
+      <c r="Q9" s="5" t="inlineStr">
+        <is>
+          <t>No government or state shareholder found in public sources</t>
+        </is>
+      </c>
+      <c r="R9" s="5" t="inlineStr">
+        <is>
+          <t>Low to medium</t>
+        </is>
+      </c>
+      <c r="S9" s="5" t="inlineStr">
+        <is>
+          <t>waffer.dhr.gov.ae (WECARE Bldg Cleaning)</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="5" t="n">
+        <v>9</v>
+      </c>
+      <c r="B10" s="8" t="inlineStr">
+        <is>
+          <t>Safaeewala Cleaning &amp; Technical Services LLC</t>
+        </is>
+      </c>
+      <c r="C10" s="5" t="inlineStr">
+        <is>
+          <t>Deep cleaning, AC maintenance, technical services</t>
+        </is>
+      </c>
+      <c r="D10" s="5" t="inlineStr">
+        <is>
+          <t>Family-run private company. Owner not published</t>
+        </is>
+      </c>
+      <c r="E10" s="5" t="inlineStr">
+        <is>
+          <t>Not published</t>
+        </is>
+      </c>
+      <c r="F10" s="5" t="inlineStr">
+        <is>
+          <t>Private family</t>
+        </is>
+      </c>
+      <c r="G10" s="5" t="inlineStr">
+        <is>
+          <t>2015</t>
+        </is>
+      </c>
+      <c r="H10" s="5" t="inlineStr">
+        <is>
+          <t>Al Qusais, Dubai</t>
+        </is>
+      </c>
+      <c r="I10" s="5" t="inlineStr">
+        <is>
+          <t>Dubai</t>
+        </is>
+      </c>
+      <c r="J10" s="5" t="inlineStr">
+        <is>
+          <t>50 to 249 (Clutch)</t>
+        </is>
+      </c>
+      <c r="K10" s="5" t="inlineStr">
+        <is>
+          <t>Residential and commercial deep cleaning</t>
+        </is>
+      </c>
+      <c r="L10" s="5" t="inlineStr">
+        <is>
+          <t>Not published</t>
+        </is>
+      </c>
+      <c r="M10" s="5" t="inlineStr">
+        <is>
+          <t>approx. AED 2M to 16M</t>
+        </is>
+      </c>
+      <c r="N10" s="5" t="inlineStr">
+        <is>
+          <t>Not published</t>
+        </is>
+      </c>
+      <c r="O10" s="5" t="inlineStr">
+        <is>
+          <t>Residential and commercial</t>
+        </is>
+      </c>
+      <c r="P10" s="5" t="inlineStr">
+        <is>
+          <t>Dubai cleaning competitor</t>
+        </is>
+      </c>
+      <c r="Q10" s="5" t="inlineStr">
+        <is>
+          <t>No government or state shareholder found in public sources</t>
+        </is>
+      </c>
+      <c r="R10" s="5" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="S10" s="5" t="inlineStr">
+        <is>
+          <t>clutch.co (Safaeewala); trustpilot.com; leadstal.com</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="5" t="n">
+        <v>10</v>
+      </c>
+      <c r="B11" s="8" t="inlineStr">
+        <is>
+          <t>EcoClean</t>
+        </is>
+      </c>
+      <c r="C11" s="5" t="inlineStr">
+        <is>
+          <t>Eco-friendly residential and commercial cleaning, AC and kitchen deep cleaning</t>
+        </is>
+      </c>
+      <c r="D11" s="5" t="inlineStr">
+        <is>
+          <t>Private. Owner not published</t>
+        </is>
+      </c>
+      <c r="E11" s="5" t="inlineStr">
+        <is>
+          <t>Not published</t>
+        </is>
+      </c>
+      <c r="F11" s="5" t="inlineStr">
+        <is>
+          <t>Private</t>
+        </is>
+      </c>
+      <c r="G11" s="5" t="inlineStr">
+        <is>
+          <t>Not reliably published</t>
+        </is>
+      </c>
+      <c r="H11" s="5" t="inlineStr">
+        <is>
+          <t>Dubai</t>
+        </is>
+      </c>
+      <c r="I11" s="5" t="inlineStr">
+        <is>
+          <t>Dubai</t>
+        </is>
+      </c>
+      <c r="J11" s="5" t="inlineStr">
+        <is>
+          <t>201 to 500 (single profile, unverified)</t>
+        </is>
+      </c>
+      <c r="K11" s="5" t="inlineStr">
+        <is>
+          <t>Heavy online marketing</t>
+        </is>
+      </c>
+      <c r="L11" s="5" t="inlineStr">
+        <is>
+          <t>Not published</t>
+        </is>
+      </c>
+      <c r="M11" s="5" t="inlineStr">
+        <is>
+          <t>Cannot estimate (headcount unknown)</t>
+        </is>
+      </c>
+      <c r="N11" s="5" t="inlineStr">
+        <is>
+          <t>Not published</t>
+        </is>
+      </c>
+      <c r="O11" s="5" t="inlineStr">
+        <is>
+          <t>Residential, holiday homes, offices</t>
+        </is>
+      </c>
+      <c r="P11" s="5" t="inlineStr">
+        <is>
+          <t>Visible Dubai cleaning brand</t>
+        </is>
+      </c>
+      <c r="Q11" s="5" t="inlineStr">
+        <is>
+          <t>No government or state shareholder found in public sources</t>
+        </is>
+      </c>
+      <c r="R11" s="5" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="S11" s="5" t="inlineStr">
+        <is>
+          <t>cyprus-mail.com; arabtimesonline.com (promotional coverage)</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="5" t="n">
+        <v>11</v>
+      </c>
+      <c r="B12" s="8" t="inlineStr">
+        <is>
+          <t>Helpsters Cleaning Services LLC</t>
+        </is>
+      </c>
+      <c r="C12" s="5" t="inlineStr">
+        <is>
+          <t>Maid service, deep cleaning, disinfection, commercial cleaning</t>
+        </is>
+      </c>
+      <c r="D12" s="5" t="inlineStr">
+        <is>
+          <t>Private. Owner not published</t>
+        </is>
+      </c>
+      <c r="E12" s="5" t="inlineStr">
+        <is>
+          <t>Not published</t>
+        </is>
+      </c>
+      <c r="F12" s="5" t="inlineStr">
+        <is>
+          <t>Private</t>
+        </is>
+      </c>
+      <c r="G12" s="5" t="inlineStr">
+        <is>
+          <t>Not published</t>
+        </is>
+      </c>
+      <c r="H12" s="5" t="inlineStr">
+        <is>
+          <t>Burj Khalifa area, Dubai</t>
+        </is>
+      </c>
+      <c r="I12" s="5" t="inlineStr">
+        <is>
+          <t>Dubai</t>
+        </is>
+      </c>
+      <c r="J12" s="5" t="inlineStr">
+        <is>
+          <t>Not published</t>
+        </is>
+      </c>
+      <c r="K12" s="5" t="inlineStr">
+        <is>
+          <t>Home and commercial</t>
+        </is>
+      </c>
+      <c r="L12" s="5" t="inlineStr">
+        <is>
+          <t>Not published</t>
+        </is>
+      </c>
+      <c r="M12" s="5" t="inlineStr">
+        <is>
+          <t>Cannot estimate (headcount unknown)</t>
+        </is>
+      </c>
+      <c r="N12" s="5" t="inlineStr">
+        <is>
+          <t>Not published</t>
+        </is>
+      </c>
+      <c r="O12" s="5" t="inlineStr">
+        <is>
+          <t>Residential and commercial</t>
+        </is>
+      </c>
+      <c r="P12" s="5" t="inlineStr">
+        <is>
+          <t>Dubai cleaning competitor</t>
+        </is>
+      </c>
+      <c r="Q12" s="5" t="inlineStr">
+        <is>
+          <t>No government or state shareholder found in public sources</t>
+        </is>
+      </c>
+      <c r="R12" s="5" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="S12" s="5" t="inlineStr">
+        <is>
+          <t>propertyfinder.ae (cleaning companies); magicpin.com</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="5" t="n">
+        <v>12</v>
+      </c>
+      <c r="B13" s="8" t="inlineStr">
+        <is>
+          <t>Urban Company UAE</t>
+        </is>
+      </c>
+      <c r="C13" s="5" t="inlineStr">
+        <is>
+          <t>App-based home cleaning (monthly subscriptions, 30-minute instant cleaning) and other home services</t>
+        </is>
+      </c>
+      <c r="D13" s="5" t="inlineStr">
+        <is>
+          <t>Urban Company Limited (India)</t>
+        </is>
+      </c>
+      <c r="E13" s="5" t="inlineStr">
+        <is>
+          <t>Indian (parent)</t>
+        </is>
+      </c>
+      <c r="F13" s="5" t="inlineStr">
+        <is>
+          <t>Private (VC-backed, IPO-bound parent)</t>
+        </is>
+      </c>
+      <c r="G13" s="5" t="inlineStr">
+        <is>
+          <t>Dubai 2018; Abu Dhabi 2019</t>
+        </is>
+      </c>
+      <c r="H13" s="5" t="inlineStr">
+        <is>
+          <t>Dubai</t>
+        </is>
+      </c>
+      <c r="I13" s="5" t="inlineStr">
+        <is>
+          <t>Dubai, Abu Dhabi, Sharjah</t>
+        </is>
+      </c>
+      <c r="J13" s="5" t="inlineStr">
+        <is>
+          <t>Not published for UAE</t>
+        </is>
+      </c>
+      <c r="K13" s="5" t="inlineStr">
+        <is>
+          <t>Also sold through the noon app</t>
+        </is>
+      </c>
+      <c r="L13" s="5" t="inlineStr">
+        <is>
+          <t>Not published for UAE</t>
+        </is>
+      </c>
+      <c r="M13" s="5" t="inlineStr">
+        <is>
+          <t>Cannot estimate (headcount unknown)</t>
+        </is>
+      </c>
+      <c r="N13" s="5" t="inlineStr">
+        <is>
+          <t>Not applicable</t>
+        </is>
+      </c>
+      <c r="O13" s="5" t="inlineStr">
+        <is>
+          <t>Residential consumers</t>
+        </is>
+      </c>
+      <c r="P13" s="5" t="inlineStr">
+        <is>
+          <t>Residential cleaning platform</t>
+        </is>
+      </c>
+      <c r="Q13" s="5" t="inlineStr">
+        <is>
+          <t>No government or state shareholder found in public sources</t>
+        </is>
+      </c>
+      <c r="R13" s="5" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="S13" s="5" t="inlineStr">
+        <is>
+          <t>urbancompany.com (Abu Dhabi launch); khaleejtimes.com (monthly subscription); gulfnews.com (noon partnership)</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="5" t="n">
+        <v>13</v>
+      </c>
+      <c r="B14" s="8" t="inlineStr">
+        <is>
+          <t>Molly Maid Dubai</t>
+        </is>
+      </c>
+      <c r="C14" s="5" t="inlineStr">
+        <is>
+          <t>Home and office cleaning</t>
+        </is>
+      </c>
+      <c r="D14" s="5" t="inlineStr">
+        <is>
+          <t>Local franchisee (not published) of Molly Maid / Neighborly (USA)</t>
+        </is>
+      </c>
+      <c r="E14" s="5" t="inlineStr">
+        <is>
+          <t>Not published</t>
+        </is>
+      </c>
+      <c r="F14" s="5" t="inlineStr">
+        <is>
+          <t>Private franchise</t>
+        </is>
+      </c>
+      <c r="G14" s="5" t="inlineStr">
+        <is>
+          <t>Approx. 25 years in Dubai (self-reported)</t>
+        </is>
+      </c>
+      <c r="H14" s="5" t="inlineStr">
+        <is>
+          <t>Dubai</t>
+        </is>
+      </c>
+      <c r="I14" s="5" t="inlineStr">
+        <is>
+          <t>Dubai</t>
+        </is>
+      </c>
+      <c r="J14" s="5" t="inlineStr">
+        <is>
+          <t>Not published</t>
+        </is>
+      </c>
+      <c r="K14" s="5" t="inlineStr">
+        <is>
+          <t>International franchise brand</t>
+        </is>
+      </c>
+      <c r="L14" s="5" t="inlineStr">
+        <is>
+          <t>Not published</t>
+        </is>
+      </c>
+      <c r="M14" s="5" t="inlineStr">
+        <is>
+          <t>Cannot estimate (headcount unknown)</t>
+        </is>
+      </c>
+      <c r="N14" s="5" t="inlineStr">
+        <is>
+          <t>Not published</t>
+        </is>
+      </c>
+      <c r="O14" s="5" t="inlineStr">
+        <is>
+          <t>Residential and offices</t>
+        </is>
+      </c>
+      <c r="P14" s="5" t="inlineStr">
+        <is>
+          <t>Branded home-cleaning competitor</t>
+        </is>
+      </c>
+      <c r="Q14" s="5" t="inlineStr">
+        <is>
+          <t>No government or state shareholder found in public sources</t>
+        </is>
+      </c>
+      <c r="R14" s="5" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="S14" s="5" t="inlineStr">
+        <is>
+          <t>business.google.com (Molly Maid Dubai); franchising.com</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="5" t="n">
+        <v>14</v>
+      </c>
+      <c r="B15" s="8" t="inlineStr">
+        <is>
+          <t>The Perfect Help (TPH Group)</t>
+        </is>
+      </c>
+      <c r="C15" s="5" t="inlineStr">
+        <is>
+          <t>Professional cleaning and maintenance</t>
+        </is>
+      </c>
+      <c r="D15" s="5" t="inlineStr">
+        <is>
+          <t>Emirati-owned and managed. Owner not published</t>
+        </is>
+      </c>
+      <c r="E15" s="5" t="inlineStr">
+        <is>
+          <t>Emirati</t>
+        </is>
+      </c>
+      <c r="F15" s="5" t="inlineStr">
+        <is>
+          <t>Private</t>
+        </is>
+      </c>
+      <c r="G15" s="5" t="inlineStr">
+        <is>
+          <t>Not published</t>
+        </is>
+      </c>
+      <c r="H15" s="5" t="inlineStr">
+        <is>
+          <t>Business Bay, Dubai</t>
+        </is>
+      </c>
+      <c r="I15" s="5" t="inlineStr">
+        <is>
+          <t>UAE</t>
+        </is>
+      </c>
+      <c r="J15" s="5" t="inlineStr">
+        <is>
+          <t>Not published</t>
+        </is>
+      </c>
+      <c r="K15" s="5" t="inlineStr">
+        <is>
+          <t>Cleaning plus AC maintenance</t>
+        </is>
+      </c>
+      <c r="L15" s="5" t="inlineStr">
+        <is>
+          <t>Not published</t>
+        </is>
+      </c>
+      <c r="M15" s="5" t="inlineStr">
+        <is>
+          <t>Cannot estimate (headcount unknown)</t>
+        </is>
+      </c>
+      <c r="N15" s="5" t="inlineStr">
+        <is>
+          <t>Not published</t>
+        </is>
+      </c>
+      <c r="O15" s="5" t="inlineStr">
+        <is>
+          <t>Not published</t>
+        </is>
+      </c>
+      <c r="P15" s="5" t="inlineStr">
+        <is>
+          <t>Emirati-owned Dubai cleaning competitor</t>
+        </is>
+      </c>
+      <c r="Q15" s="5" t="inlineStr">
+        <is>
+          <t>No government or state shareholder found in public sources</t>
+        </is>
+      </c>
+      <c r="R15" s="5" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="S15" s="5" t="inlineStr">
+        <is>
+          <t>naukrigulf.com (TPH Group); ae.indeed.com</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="5" t="n">
+        <v>15</v>
+      </c>
+      <c r="B16" s="8" t="inlineStr">
+        <is>
+          <t>Schon Building Cleaning Services LLC</t>
+        </is>
+      </c>
+      <c r="C16" s="5" t="inlineStr">
+        <is>
+          <t>Commercial cleaning, deep cleaning, sanitisation</t>
+        </is>
+      </c>
+      <c r="D16" s="5" t="inlineStr">
+        <is>
+          <t>Private. Owner not published</t>
+        </is>
+      </c>
+      <c r="E16" s="5" t="inlineStr">
+        <is>
+          <t>Not published</t>
+        </is>
+      </c>
+      <c r="F16" s="5" t="inlineStr">
+        <is>
+          <t>Private</t>
+        </is>
+      </c>
+      <c r="G16" s="5" t="inlineStr">
+        <is>
+          <t>2017</t>
+        </is>
+      </c>
+      <c r="H16" s="5" t="inlineStr">
+        <is>
+          <t>Dubai</t>
+        </is>
+      </c>
+      <c r="I16" s="5" t="inlineStr">
+        <is>
+          <t>Dubai</t>
+        </is>
+      </c>
+      <c r="J16" s="5" t="inlineStr">
+        <is>
+          <t>11 to 50 (directory)</t>
+        </is>
+      </c>
+      <c r="K16" s="5" t="inlineStr">
+        <is>
+          <t>Small commercial cleaner</t>
+        </is>
+      </c>
+      <c r="L16" s="5" t="inlineStr">
+        <is>
+          <t>Not published</t>
+        </is>
+      </c>
+      <c r="M16" s="5" t="inlineStr">
+        <is>
+          <t>approx. AED 0M to 3M</t>
+        </is>
+      </c>
+      <c r="N16" s="5" t="inlineStr">
+        <is>
+          <t>Not published</t>
+        </is>
+      </c>
+      <c r="O16" s="5" t="inlineStr">
+        <is>
+          <t>Commercial</t>
+        </is>
+      </c>
+      <c r="P16" s="5" t="inlineStr">
+        <is>
+          <t>Dubai commercial cleaning competitor</t>
+        </is>
+      </c>
+      <c r="Q16" s="5" t="inlineStr">
+        <is>
+          <t>No government or state shareholder found in public sources</t>
+        </is>
+      </c>
+      <c r="R16" s="5" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="S16" s="5" t="inlineStr">
+        <is>
+          <t>ensun.io (commercial cleaning UAE)</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="5" t="n">
+        <v>16</v>
+      </c>
+      <c r="B17" s="8" t="inlineStr">
+        <is>
+          <t>CleaningCompany.ae</t>
+        </is>
+      </c>
+      <c r="C17" s="5" t="inlineStr">
+        <is>
+          <t>Residential and commercial cleaning</t>
+        </is>
+      </c>
+      <c r="D17" s="5" t="inlineStr">
+        <is>
+          <t>Private. Owner not published</t>
+        </is>
+      </c>
+      <c r="E17" s="5" t="inlineStr">
+        <is>
+          <t>Not published</t>
+        </is>
+      </c>
+      <c r="F17" s="5" t="inlineStr">
+        <is>
+          <t>Private</t>
+        </is>
+      </c>
+      <c r="G17" s="5" t="inlineStr">
+        <is>
+          <t>Not published</t>
+        </is>
+      </c>
+      <c r="H17" s="5" t="inlineStr">
+        <is>
+          <t>Dubai</t>
+        </is>
+      </c>
+      <c r="I17" s="5" t="inlineStr">
+        <is>
+          <t>UAE</t>
+        </is>
+      </c>
+      <c r="J17" s="5" t="inlineStr">
+        <is>
+          <t>Not published</t>
+        </is>
+      </c>
+      <c r="K17" s="5" t="inlineStr">
+        <is>
+          <t>Featured by Gulf News as a start-up to watch</t>
+        </is>
+      </c>
+      <c r="L17" s="5" t="inlineStr">
+        <is>
+          <t>Not published</t>
+        </is>
+      </c>
+      <c r="M17" s="5" t="inlineStr">
+        <is>
+          <t>Cannot estimate (headcount unknown)</t>
+        </is>
+      </c>
+      <c r="N17" s="5" t="inlineStr">
+        <is>
+          <t>Not published</t>
+        </is>
+      </c>
+      <c r="O17" s="5" t="inlineStr">
+        <is>
+          <t>Residential and commercial</t>
+        </is>
+      </c>
+      <c r="P17" s="5" t="inlineStr">
+        <is>
+          <t>Dubai cleaning competitor</t>
+        </is>
+      </c>
+      <c r="Q17" s="5" t="inlineStr">
+        <is>
+          <t>No government or state shareholder found in public sources</t>
+        </is>
+      </c>
+      <c r="R17" s="5" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="S17" s="5" t="inlineStr">
+        <is>
+          <t>gulfnews.com ('A start-up to look out for in Dubai'); sothebysrealty.ae</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="5" t="n">
+        <v>17</v>
+      </c>
+      <c r="B18" s="8" t="inlineStr">
+        <is>
+          <t>Bookaclean</t>
+        </is>
+      </c>
+      <c r="C18" s="5" t="inlineStr">
+        <is>
+          <t>Residential and commercial cleaning with flexible booking</t>
+        </is>
+      </c>
+      <c r="D18" s="5" t="inlineStr">
+        <is>
+          <t>Ploesteanca Dumitrascu (per company press release, unverified)</t>
+        </is>
+      </c>
+      <c r="E18" s="5" t="inlineStr">
+        <is>
+          <t>Not published</t>
+        </is>
+      </c>
+      <c r="F18" s="5" t="inlineStr">
+        <is>
+          <t>Private</t>
+        </is>
+      </c>
+      <c r="G18" s="5" t="inlineStr">
+        <is>
+          <t>Not published</t>
+        </is>
+      </c>
+      <c r="H18" s="5" t="inlineStr">
+        <is>
+          <t>Dubai</t>
+        </is>
+      </c>
+      <c r="I18" s="5" t="inlineStr">
+        <is>
+          <t>Dubai</t>
+        </is>
+      </c>
+      <c r="J18" s="5" t="inlineStr">
+        <is>
+          <t>Not published</t>
+        </is>
+      </c>
+      <c r="K18" s="5" t="inlineStr">
+        <is>
+          <t>Online booking</t>
+        </is>
+      </c>
+      <c r="L18" s="5" t="inlineStr">
+        <is>
+          <t>Not published</t>
+        </is>
+      </c>
+      <c r="M18" s="5" t="inlineStr">
+        <is>
+          <t>Cannot estimate (headcount unknown)</t>
+        </is>
+      </c>
+      <c r="N18" s="5" t="inlineStr">
+        <is>
+          <t>Not published</t>
+        </is>
+      </c>
+      <c r="O18" s="5" t="inlineStr">
+        <is>
+          <t>Residential and commercial</t>
+        </is>
+      </c>
+      <c r="P18" s="5" t="inlineStr">
+        <is>
+          <t>Dubai cleaning competitor</t>
+        </is>
+      </c>
+      <c r="Q18" s="5" t="inlineStr">
+        <is>
+          <t>No government or state shareholder found in public sources</t>
+        </is>
+      </c>
+      <c r="R18" s="5" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="S18" s="5" t="inlineStr">
+        <is>
+          <t>markets.financialcontent.com (ACCESS Newswire release); eyeofriyadh.com</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="5" t="n">
+        <v>18</v>
+      </c>
+      <c r="B19" s="8" t="inlineStr">
+        <is>
+          <t>Helpbit Homes</t>
+        </is>
+      </c>
+      <c r="C19" s="5" t="inlineStr">
+        <is>
+          <t>Home and office cleaning, pest control, moving, at-home salon</t>
+        </is>
+      </c>
+      <c r="D19" s="5" t="inlineStr">
+        <is>
+          <t>Private. Owner not published</t>
+        </is>
+      </c>
+      <c r="E19" s="5" t="inlineStr">
+        <is>
+          <t>Not published</t>
+        </is>
+      </c>
+      <c r="F19" s="5" t="inlineStr">
+        <is>
+          <t>Private</t>
+        </is>
+      </c>
+      <c r="G19" s="5" t="inlineStr">
+        <is>
+          <t>Not published</t>
+        </is>
+      </c>
+      <c r="H19" s="5" t="inlineStr">
+        <is>
+          <t>Dubai</t>
+        </is>
+      </c>
+      <c r="I19" s="5" t="inlineStr">
+        <is>
+          <t>Dubai</t>
+        </is>
+      </c>
+      <c r="J19" s="5" t="inlineStr">
+        <is>
+          <t>Not published</t>
+        </is>
+      </c>
+      <c r="K19" s="5" t="inlineStr">
+        <is>
+          <t>Multi-service home platform</t>
+        </is>
+      </c>
+      <c r="L19" s="5" t="inlineStr">
+        <is>
+          <t>Not published</t>
+        </is>
+      </c>
+      <c r="M19" s="5" t="inlineStr">
+        <is>
+          <t>Cannot estimate (headcount unknown)</t>
+        </is>
+      </c>
+      <c r="N19" s="5" t="inlineStr">
+        <is>
+          <t>Not published</t>
+        </is>
+      </c>
+      <c r="O19" s="5" t="inlineStr">
+        <is>
+          <t>Residential and offices</t>
+        </is>
+      </c>
+      <c r="P19" s="5" t="inlineStr">
+        <is>
+          <t>Residential cleaning competitor</t>
+        </is>
+      </c>
+      <c r="Q19" s="5" t="inlineStr">
+        <is>
+          <t>No government or state shareholder found in public sources</t>
+        </is>
+      </c>
+      <c r="R19" s="5" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="S19" s="5" t="inlineStr">
+        <is>
+          <t>mustakbil.com (Helpbit Homes); squareyards.ae</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="5" t="n">
+        <v>19</v>
+      </c>
+      <c r="B20" s="8" t="inlineStr">
+        <is>
+          <t>Hello Cleaner</t>
+        </is>
+      </c>
+      <c r="C20" s="5" t="inlineStr">
+        <is>
+          <t>Home and office cleaning</t>
+        </is>
+      </c>
+      <c r="D20" s="5" t="inlineStr">
+        <is>
+          <t>Private. Owner not published</t>
+        </is>
+      </c>
+      <c r="E20" s="5" t="inlineStr">
+        <is>
+          <t>Not published</t>
+        </is>
+      </c>
+      <c r="F20" s="5" t="inlineStr">
+        <is>
+          <t>Private</t>
+        </is>
+      </c>
+      <c r="G20" s="5" t="inlineStr">
+        <is>
+          <t>Not published</t>
+        </is>
+      </c>
+      <c r="H20" s="5" t="inlineStr">
+        <is>
+          <t>Dubai</t>
+        </is>
+      </c>
+      <c r="I20" s="5" t="inlineStr">
+        <is>
+          <t>Dubai</t>
+        </is>
+      </c>
+      <c r="J20" s="5" t="inlineStr">
+        <is>
+          <t>Not published</t>
+        </is>
+      </c>
+      <c r="K20" s="5" t="inlineStr">
+        <is>
+          <t>92 salary reviews on Indeed</t>
+        </is>
+      </c>
+      <c r="L20" s="5" t="inlineStr">
+        <is>
+          <t>Not published</t>
+        </is>
+      </c>
+      <c r="M20" s="5" t="inlineStr">
+        <is>
+          <t>Cannot estimate (headcount unknown)</t>
+        </is>
+      </c>
+      <c r="N20" s="5" t="inlineStr">
+        <is>
+          <t>Not published</t>
+        </is>
+      </c>
+      <c r="O20" s="5" t="inlineStr">
+        <is>
+          <t>Residential and offices</t>
+        </is>
+      </c>
+      <c r="P20" s="5" t="inlineStr">
+        <is>
+          <t>Dubai cleaning competitor</t>
+        </is>
+      </c>
+      <c r="Q20" s="5" t="inlineStr">
+        <is>
+          <t>No government or state shareholder found in public sources</t>
+        </is>
+      </c>
+      <c r="R20" s="5" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="S20" s="5" t="inlineStr">
+        <is>
+          <t>ae.indeed.com (Hello Cleaner); crunchbase.com</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="5" t="n">
+        <v>20</v>
+      </c>
+      <c r="B21" s="8" t="inlineStr">
+        <is>
+          <t>Home Maids</t>
+        </is>
+      </c>
+      <c r="C21" s="5" t="inlineStr">
+        <is>
+          <t>Hourly maid and home cleaning services</t>
+        </is>
+      </c>
+      <c r="D21" s="5" t="inlineStr">
+        <is>
+          <t>Private. Owner not published</t>
+        </is>
+      </c>
+      <c r="E21" s="5" t="inlineStr">
+        <is>
+          <t>Not published</t>
+        </is>
+      </c>
+      <c r="F21" s="5" t="inlineStr">
+        <is>
+          <t>Private</t>
+        </is>
+      </c>
+      <c r="G21" s="5" t="inlineStr">
+        <is>
+          <t>2005</t>
+        </is>
+      </c>
+      <c r="H21" s="5" t="inlineStr">
+        <is>
+          <t>Dubai</t>
+        </is>
+      </c>
+      <c r="I21" s="5" t="inlineStr">
+        <is>
+          <t>Dubai</t>
+        </is>
+      </c>
+      <c r="J21" s="5" t="inlineStr">
+        <is>
+          <t>Not published</t>
+        </is>
+      </c>
+      <c r="K21" s="5" t="inlineStr">
+        <is>
+          <t>Hourly maid supply</t>
+        </is>
+      </c>
+      <c r="L21" s="5" t="inlineStr">
+        <is>
+          <t>Not published</t>
+        </is>
+      </c>
+      <c r="M21" s="5" t="inlineStr">
+        <is>
+          <t>Cannot estimate (headcount unknown)</t>
+        </is>
+      </c>
+      <c r="N21" s="5" t="inlineStr">
+        <is>
+          <t>Not published</t>
+        </is>
+      </c>
+      <c r="O21" s="5" t="inlineStr">
+        <is>
+          <t>Residential</t>
+        </is>
+      </c>
+      <c r="P21" s="5" t="inlineStr">
+        <is>
+          <t>Residential cleaning competitor</t>
+        </is>
+      </c>
+      <c r="Q21" s="5" t="inlineStr">
+        <is>
+          <t>No government or state shareholder found in public sources</t>
+        </is>
+      </c>
+      <c r="R21" s="5" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="S21" s="5" t="inlineStr">
+        <is>
+          <t>khaleejtimes.com ('Home maids in Dubai')</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:S7"/>
+  <autoFilter ref="A1:S21"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -3033,7 +6833,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B16"/>
+  <dimension ref="A1:B27"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -3232,6 +7032,138 @@
         </is>
       </c>
     </row>
+    <row r="17">
+      <c r="A17" s="11" t="inlineStr">
+        <is>
+          <t>Khadamat Facilities Management</t>
+        </is>
+      </c>
+      <c r="B17" s="5" t="inlineStr">
+        <is>
+          <t>Set up as a JV of Mubadala (Abu Dhabi state investor) and Serco</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="11" t="inlineStr">
+        <is>
+          <t>Ontegra (formerly Deyaar FM)</t>
+        </is>
+      </c>
+      <c r="B18" s="5" t="inlineStr">
+        <is>
+          <t>Subsidiary of Deyaar Development (government-linked)</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="11" t="inlineStr">
+        <is>
+          <t>Tafawuq Facility Management</t>
+        </is>
+      </c>
+      <c r="B19" s="5" t="inlineStr">
+        <is>
+          <t>Owned by Eltizam, which is 50% ADQ (Abu Dhabi state holding) and 50% IHC</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="11" t="inlineStr">
+        <is>
+          <t>Emirates International Facility Management</t>
+        </is>
+      </c>
+      <c r="B20" s="5" t="inlineStr">
+        <is>
+          <t>Subsidiary of Das Holding, reported to be owned by Sheikh Mansour bin Zayed</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="11" t="inlineStr">
+        <is>
+          <t>Operon Middle East</t>
+        </is>
+      </c>
+      <c r="B21" s="5" t="inlineStr">
+        <is>
+          <t>Owned by Edgenta, part of UEM Group, which belongs to Malaysia's state fund Khazanah</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="11" t="inlineStr">
+        <is>
+          <t>Spark Security Services</t>
+        </is>
+      </c>
+      <c r="B22" s="5" t="inlineStr">
+        <is>
+          <t>Acquired by Aldar Properties in 2022</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="11" t="inlineStr">
+        <is>
+          <t>World Security</t>
+        </is>
+      </c>
+      <c r="B23" s="5" t="inlineStr">
+        <is>
+          <t>Owned by DP World (Dubai Government)</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="11" t="inlineStr">
+        <is>
+          <t>GardaWorld UAE</t>
+        </is>
+      </c>
+      <c r="B24" s="5" t="inlineStr">
+        <is>
+          <t>Operates in the UAE through a joint venture with Transguard</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="11" t="inlineStr">
+        <is>
+          <t>Global Security Services Group (GSSG)</t>
+        </is>
+      </c>
+      <c r="B25" s="5" t="inlineStr">
+        <is>
+          <t>Describes itself as the armed security provider for the UAE government</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="11" t="inlineStr">
+        <is>
+          <t>Duserve FM &amp; Building Cleaning</t>
+        </is>
+      </c>
+      <c r="B26" s="5" t="inlineStr">
+        <is>
+          <t>Owned by Dubai World Central (Government of Dubai)</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="11" t="inlineStr">
+        <is>
+          <t>Hitches &amp; Glitches</t>
+        </is>
+      </c>
+      <c r="B27" s="5" t="inlineStr">
+        <is>
+          <t>Not separate: a subsidiary of Farnek, which is already listed</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>